<commit_message>
Libretto Manuel: voci più sintetiche e ore stimate
Descrizioni ridotte a una frase, percorsi dei file aggiornati a quelli
attuali e una stima di ore per ogni voce (25 ore in tutto, al massimo
circa 9 ore in un giorno).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/libretti/manuel-bulla.xlsx
+++ b/docs/libretti/manuel-bulla.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bulla\AppData\Local\Temp\claude\C--Users-bulla-Documents-Ing-software-v1\c32cf868-ae9e-4ff3-a799-856eab5b1d43\scratchpad\out\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bulla\Documents\Ing-software-v1\docs\libretti\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C878ED29-E396-4254-83AE-A2FD767EA069}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBAB41D6-2505-4458-9767-AAF41C4AF7CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{EB300ADB-58B5-479D-B51B-E912DFEACD78}"/>
   </bookViews>
@@ -84,168 +84,93 @@
     <t>Avvio repository</t>
   </si>
   <si>
-    <t>Creazione del repository GitHub del progetto, primo commit e collegamento al remote origin.</t>
-  </si>
-  <si>
     <t>Ing-software-prog-test-v1</t>
   </si>
   <si>
     <t>Prima versione presentazione</t>
   </si>
   <si>
-    <t>Caricata nel repository la prima versione della presentazione del progetto (5 slide: contesto, problema, soluzione, vantaggi).</t>
-  </si>
-  <si>
-    <t>DISCOVER_TRIDENTUM_VF.pptx</t>
-  </si>
-  <si>
     <t>Nuovo design presentazione</t>
   </si>
   <si>
-    <t>Revisione della presentazione: design più pulito e testi più sintetici, dettagli spostati nelle note del relatore.</t>
-  </si>
-  <si>
-    <t>DISCOVER_TRIDENTUM_v2.pptx</t>
-  </si>
-  <si>
     <t>Organizzazione repository</t>
   </si>
   <si>
-    <t>Creata la cartella presentazioni/ e spostati i file; integrate le modifiche dei compagni (git pull --rebase) prima del push.</t>
-  </si>
-  <si>
     <t>presentazioni/</t>
   </si>
   <si>
     <t>README del progetto</t>
   </si>
   <si>
-    <t>Scrittura del README GitHub: descrizione, problema, funzionalità, stakeholder, struttura del repository, team.</t>
-  </si>
-  <si>
     <t>README.md</t>
   </si>
   <si>
     <t>Fase 1 — Analisi del dominio</t>
   </si>
   <si>
-    <t>Documento di Fase 1: analisi del dominio, 2 personas (turista e residente), Stakeholder Matrix interesse/potere, matrice di tracciabilità problema → bisogno → requisito.</t>
-  </si>
-  <si>
     <t>docs/fase-1-analisi-dominio.md</t>
   </si>
   <si>
     <t>Libretti delle attività</t>
   </si>
   <si>
-    <t>Creata la cartella documentazione/ con un libretto delle attività per ciascun membro del team.</t>
-  </si>
-  <si>
-    <t>documentazione/</t>
-  </si>
-  <si>
     <t>Fase 2 — Specifiche dei requisiti</t>
   </si>
   <si>
-    <t>SRS Light: 29 requisiti funzionali prioritizzati con MoSCoW (11 Must, 9 Should, 5 Could, 4 Won't), requisiti non funzionali (usabilità, prestazioni, sicurezza, portabilità) con metriche, 7 casi d'uso con diagramma.</t>
-  </si>
-  <si>
     <t>docs/fase-2-specifiche-requisiti.md</t>
   </si>
   <si>
     <t>Riorganizzazione secondo le convenzioni</t>
   </si>
   <si>
-    <t>Revisione del repository: cartelle e nomi dei file uniformati (documentazione/ → docs/libretti/, presentazioni rinominate in presentazione-v1/v2, proposta PDF in docs/fase-0-proposta-progetto.pdf); aggiunti .gitignore, .gitattributes e CONTRIBUTING.md con le convenzioni del team; Fase 1 e Fase 2 portate alla versione 0.2 con storico delle revisioni e matrice di tracciabilità (vecchi → nuovi ID, bisogni → requisiti, requisiti → casi d'uso).</t>
-  </si>
-  <si>
     <t>CONTRIBUTING.md, docs/</t>
   </si>
   <si>
     <t>Pubblicazione della riorganizzazione</t>
   </si>
   <si>
-    <t>Commit e push su GitHub della riorganizzazione del repository (commit 34fe9ee), dopo git pull --rebase per integrare eventuali modifiche dei compagni. Aggiornato il libretto con le attività svolte.</t>
-  </si>
-  <si>
     <t>main su GitHub</t>
   </si>
   <si>
     <t>Fase 3 — Architettura e user flow</t>
   </si>
   <si>
-    <t>Documento di Fase 3: diagramma dei casi d'uso in Mermaid (vista generale e relazioni «include»/«extend»), elenco delle schermate, flusso dall'accesso alla consultazione, mappa di navigazione, user journey delle personas, architettura ad alto livello (Frontend Web, API Gateway, Backend, AI Service, Database, Storage foto), decisioni architetturali, diagrammi di sequenza, deployment e tracciabilità. Fase 2 aggiornata alla v0.3 con i casi d'uso UC-08, UC-09, UC-10. Diagrammi verificati con il renderer Mermaid.</t>
-  </si>
-  <si>
     <t>docs/fase-3-architettura-user-flow.md</t>
   </si>
   <si>
     <t>Fase 4 — Pianificazione dello sviluppo</t>
   </si>
   <si>
-    <t>Documento di Fase 4: definizione dell'MVP con ordine di taglio dei requisiti Should, WBS in 11 pacchetti e 43 task stimati (261 h), percorso critico, capacità del team, piano con Sprint 0, tre sprint da 3 settimane e stabilizzazione, roadmap Gantt con 5 milestone (MVP entro il 20/12/2026), processo Scrum semplificato e Definition of Done, matrice dei rischi tecnici e di progetto (15 rischi) con prevenzione, piano B e indicatori. Diagrammi verificati con il renderer Mermaid.</t>
-  </si>
-  <si>
     <t>docs/fase-4-pianificazione.md</t>
   </si>
   <si>
     <t>Revisione della pianificazione</t>
   </si>
   <si>
-    <t>Piano di sviluppo riorganizzato con priorità ai luoghi: ricerca, filtri e itinerari tematici portati a Must, gioco "Dov'era?" portato a Could. Fase 4 v0.2: Sprint 1 dedicato a mappa, schede e contenuti (almeno 30 POI e 15 affreschi con revisione delle fonti), Sprint 2 a gestione dei luoghi, account e itinerari, Sprint 3 alla community; il gioco è l'ultimo blocco e il primo da tagliare. Aggiunto il rischio R-16. Fase 2 aggiornata alla v0.4.</t>
-  </si>
-  <si>
     <t>docs/fase-4-pianificazione.md, docs/fase-2-specifiche-requisiti.md</t>
   </si>
   <si>
     <t>Frontend v2 e gioco fotografico</t>
   </si>
   <si>
-    <t>Nuova versione del sito in src/frontend-v2 (npm run dev:v2), costruita sulla v1 collegata al backend: mappa dei luoghi con raggruppamento dei POI vicini, icone di categoria, nomi visibili ingrandendo e sfondo attenuato; layout desktop con elenco e mappa affiancati, scheda su due colonne; copertine con il ritaglio della mappa; nuovo stile (font Geist, icone Phosphor, tema chiaro e scuro). Gioco "Dov'era?" trasformato in stile GeoGuessr: 8 foto storiche di pubblico dominio da Wikimedia Commons al posto degli indizi testuali, con crediti mostrati dopo la risposta (backend: migrazione 002, nuova rotta per le foto, test). Controllo con le Web Interface Guidelines e correzioni (accessibilità da tastiera del gioco, link veri, tipografia, titoli di pagina).</t>
-  </si>
-  <si>
-    <t>src/frontend-v2/, src/backend/src/db/dati/foto-gioco/</t>
-  </si>
-  <si>
     <t>Frontend v2 per smartphone</t>
   </si>
   <si>
-    <t>Revisione della v2 per chi la usa dal telefono: anteprima dei luoghi come pannello dal basso che si chiude trascinandolo, con la mappa che sposta il luogo selezionato nello spazio libero; scheda riordinata (informazioni pratiche e luoghi vicini prima delle fonti) con barra in alto per tornare indietro e condividere il luogo; barra fissa con le tappe dell'itinerario sopra la navigazione; avvisi sulla posizione che si chiudono da soli; aree di tocco di almeno 44 px, campi a 16 px per evitare lo zoom su iPhone, niente effetti hover dopo il tocco; vibrazione quando si mette il segnaposto nel gioco.</t>
-  </si>
-  <si>
-    <t>src/frontend-v2/</t>
-  </si>
-  <si>
     <t>Pulizia dello spazio di lavoro</t>
   </si>
   <si>
-    <t>Riordino delle cartelle dopo la separazione della versione corrente dalle versioni precedenti: rimossa la cartella src/ rimasta dal vecchio layout (build, cache e un vecchio database di prova), chiusi i server di sviluppo ancora avviati da lì, ricollegate le dipendenze dei workspace a versione-corrente/ e rieseguiti i test (7 del frontend e 146 del backend, tutti superati). Eliminato il branch locale già unito a main. La struttura del repository è stata verificata rispetto al README.</t>
-  </si>
-  <si>
-    <t>Spazio di lavoro locale; struttura del README invariata</t>
-  </si>
-  <si>
     <t>Controllo dei requisiti della Fase 2</t>
   </si>
   <si>
-    <t>Verifica della versione corrente del sito rispetto ai requisiti della Fase 2 (v0.4): requisiti funzionali e non funzionali, casi d'uso con flussi alternativi ed eccezioni. Lettura del codice di frontend e backend, esecuzione dei test (7 del frontend e 146 del backend, tutti superati), prove a 360 px di larghezza e in assenza di connessione, build di produzione. Risultato raccolto in un nuovo documento: i requisiti funzionali Must e Should sono tutti presenti; mancano o sono incompleti l'informativa privacy, la configurazione HTTPS, parte delle eccezioni dei casi d'uso, le foto dei luoghi e alcuni requisiti Could.</t>
-  </si>
-  <si>
     <t>docs/cose-mancanti.md</t>
   </si>
   <si>
     <t>Secondo controllo dei requisiti della Fase 2</t>
   </si>
   <si>
-    <t>Nuova verifica della versione corrente (frontend v3) dopo il completamento dei punti del documento Cose mancanti: lettura delle modifiche, test (11 del frontend e 274 del backend, tutti superati), prove a 360 px di larghezza, senza connessione e con Chrome (installazione come app, apertura senza rete, tempi su rete simulata, mappa allargata). Il documento è passato alla versione 0.2: 17 voci su 26 risultano chiuse; restano le foto dei luoghi (lo script di scaricamento va eseguito e la scelta rivista), i compiti del titolare per la privacy, la verifica con la Soprintendenza e le prove con persone e dispositivi reali.</t>
-  </si>
-  <si>
     <t>Libretti in Excel con conta ore</t>
   </si>
   <si>
-    <t>Convertiti i tre libretti da Word a Excel, un file per ogni membro del team: stessa tabella di prima con in più la colonna Ore, il totale delle ore, il conteggio delle voci senza ore e un riepilogo delle ore per settimana che si aggiorna da solo. Le ore delle attività già registrate non erano annotate e restano da inserire. Aggiornati CONTRIBUTING.md e .gitattributes per il nuovo formato.</t>
-  </si>
-  <si>
     <t>docs/libretti/*.xlsx</t>
   </si>
   <si>
@@ -277,6 +202,81 @@
   </si>
   <si>
     <t>Se 'Fuori dalle settimane elencate' non è zero, ci sono voci con una data oltre l'ultima settimana: inserisci una riga sopra l'ultima settimana e copia le formule dalla riga precedente.</t>
+  </si>
+  <si>
+    <t>Creato il repository GitHub, primo commit e collegamento al remote.</t>
+  </si>
+  <si>
+    <t>Prima versione della presentazione (5 slide: contesto, problema, soluzione, vantaggi).</t>
+  </si>
+  <si>
+    <t>presentazioni/presentazione-v1.pptx</t>
+  </si>
+  <si>
+    <t>Design più pulito e testi più sintetici, con i dettagli spostati nelle note del relatore.</t>
+  </si>
+  <si>
+    <t>presentazioni/presentazione-v2.pptx</t>
+  </si>
+  <si>
+    <t>Creata la cartella presentazioni/ e spostati i file; integrate le modifiche dei compagni con git pull --rebase.</t>
+  </si>
+  <si>
+    <t>README GitHub con descrizione, problema, funzionalità, stakeholder, struttura del repository e team.</t>
+  </si>
+  <si>
+    <t>Analisi del dominio, 2 personas, Stakeholder Matrix e matrice di tracciabilità problema → bisogno → requisito.</t>
+  </si>
+  <si>
+    <t>Creato un libretto delle attività per ogni membro del team.</t>
+  </si>
+  <si>
+    <t>docs/libretti/</t>
+  </si>
+  <si>
+    <t>SRS Light: 29 requisiti funzionali con MoSCoW, requisiti non funzionali con metriche e 7 casi d'uso con diagramma.</t>
+  </si>
+  <si>
+    <t>Cartelle e nomi dei file uniformati; aggiunti .gitignore, .gitattributes e CONTRIBUTING.md; Fase 1 e Fase 2 portate alla v0.2 con storico e tracciabilità.</t>
+  </si>
+  <si>
+    <t>Commit e push su GitHub dopo git pull --rebase per integrare le modifiche dei compagni.</t>
+  </si>
+  <si>
+    <t>Casi d'uso in Mermaid, schermate e flusso di navigazione, user journey, architettura ad alto livello, diagrammi di sequenza e deployment; Fase 2 alla v0.3.</t>
+  </si>
+  <si>
+    <t>Definizione dell'MVP, WBS in 11 pacchetti e 43 task (261 h), piano a sprint, roadmap con 5 milestone e matrice di 15 rischi.</t>
+  </si>
+  <si>
+    <t>Priorità ai luoghi (ricerca, filtri e itinerari a Must) e gioco "Dov'era?" a Could, come ultimo blocco; Fase 4 v0.2 e Fase 2 v0.4.</t>
+  </si>
+  <si>
+    <t>Nuovo frontend con mappa dei luoghi, layout desktop e nuovo stile; gioco "Dov'era?" in stile GeoGuessr con 8 foto storiche di pubblico dominio e relativi crediti.</t>
+  </si>
+  <si>
+    <t>versioni-precedenti/frontend-v2/, versione-corrente/backend/src/db/dati/foto-gioco/</t>
+  </si>
+  <si>
+    <t>Revisione per il telefono: anteprima dei luoghi a pannello dal basso, scheda riordinata, tappe dell'itinerario in barra fissa e aree di tocco da 44 px.</t>
+  </si>
+  <si>
+    <t>versioni-precedenti/frontend-v2/</t>
+  </si>
+  <si>
+    <t>Rimossa la cartella src/ rimasta dal vecchio layout, ricollegate le dipendenze e rieseguiti i test (tutti superati).</t>
+  </si>
+  <si>
+    <t>Spazio di lavoro locale</t>
+  </si>
+  <si>
+    <t>Verifica del sito rispetto ai requisiti della Fase 2 (codice, test, prove a 360 px e offline): Must e Should presenti, restano privacy, HTTPS e alcune eccezioni dei casi d'uso.</t>
+  </si>
+  <si>
+    <t>Nuova verifica dopo il completamento dei punti (test, prove a 360 px, offline e con Chrome): 17 voci su 26 risultano chiuse.</t>
+  </si>
+  <si>
+    <t>Libretti convertiti da Word a Excel, uno per membro, con colonna Ore, totali e riepilogo per settimana; aggiornati CONTRIBUTING.md e .gitattributes.</t>
   </si>
 </sst>
 </file>
@@ -444,74 +444,74 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -534,7 +534,7 @@
     </dxf>
     <dxf>
       <font>
-        <b/>
+        <b val="0"/>
         <i val="0"/>
         <strike val="0"/>
         <condense val="0"/>
@@ -544,18 +544,31 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
+        <color theme="1"/>
         <name val="Arial"/>
         <family val="2"/>
         <scheme val="none"/>
       </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FF1B2428"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -576,25 +589,6 @@
       </font>
       <numFmt numFmtId="164" formatCode="0.0"/>
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -652,11 +646,11 @@
         <family val="2"/>
         <scheme val="none"/>
       </font>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
-        <b val="0"/>
+        <b/>
         <i val="0"/>
         <strike val="0"/>
         <condense val="0"/>
@@ -666,12 +660,37 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="10"/>
-        <color theme="1"/>
+        <color rgb="FFFFFFFF"/>
         <name val="Arial"/>
         <family val="2"/>
         <scheme val="none"/>
       </font>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF1B2428"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFBF8F3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FFFFFFFF"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF1B2428"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <border>
@@ -695,31 +714,12 @@
         </horizontal>
       </border>
     </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFBF8F3"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFFFFFFF"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF1B2428"/>
-        </patternFill>
-      </fill>
-    </dxf>
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
     <tableStyle name="Libretto" pivot="0" count="3" xr9:uid="{4D784E34-38D5-4852-9B7C-8838ED6D73F1}">
-      <tableStyleElement type="wholeTable" dxfId="9"/>
-      <tableStyleElement type="headerRow" dxfId="11"/>
-      <tableStyleElement type="firstRowStripe" dxfId="10"/>
+      <tableStyleElement type="wholeTable" dxfId="11"/>
+      <tableStyleElement type="headerRow" dxfId="10"/>
+      <tableStyleElement type="firstRowStripe" dxfId="9"/>
     </tableStyle>
   </tableStyles>
   <extLst>
@@ -734,7 +734,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F7E690B7-EC62-4BC2-A27A-E592475A3F24}" name="Registro" displayName="Registro" ref="A8:E27" totalsRowShown="0" headerRowDxfId="2" dataDxfId="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F7E690B7-EC62-4BC2-A27A-E592475A3F24}" name="Registro" displayName="Registro" ref="A8:E27" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
   <autoFilter ref="A8:E27" xr:uid="{F7E690B7-EC62-4BC2-A27A-E592475A3F24}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -745,9 +745,9 @@
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{586C618C-B2D4-4DF9-B7CA-43309990EE13}" name="Data" dataDxfId="6"/>
     <tableColumn id="2" xr3:uid="{25096E78-7995-48E9-AD81-04E6781C948E}" name="Attività" dataDxfId="5"/>
-    <tableColumn id="3" xr3:uid="{47CC29D8-54BC-4349-A4AF-A8DBA19285A8}" name="Ore" dataDxfId="3"/>
-    <tableColumn id="4" xr3:uid="{FBB4DA33-A195-4C3A-A982-31970BE0195C}" name="Descrizione" dataDxfId="4"/>
-    <tableColumn id="5" xr3:uid="{9CC3C245-FBDD-4A24-9A04-CA85BD0504F4}" name="Risultato / file" dataDxfId="7"/>
+    <tableColumn id="3" xr3:uid="{47CC29D8-54BC-4349-A4AF-A8DBA19285A8}" name="Ore" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{FBB4DA33-A195-4C3A-A982-31970BE0195C}" name="Descrizione" dataDxfId="3"/>
+    <tableColumn id="5" xr3:uid="{9CC3C245-FBDD-4A24-9A04-CA85BD0504F4}" name="Risultato / file" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="Libretto" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1110,7 +1110,7 @@
       </c>
       <c r="C5" s="7">
         <f>SUM(Registro[Ore])</f>
-        <v>0</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="13.15" x14ac:dyDescent="0.4">
@@ -1119,318 +1119,356 @@
       </c>
       <c r="C6" s="8">
         <f>COUNTIFS(Registro[Attività],"&lt;&gt;",Registro[Ore],"")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="31" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" s="32"/>
+      <c r="C7" s="32"/>
+      <c r="D7" s="32"/>
+      <c r="E7" s="32"/>
+    </row>
+    <row r="8" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8" s="14" t="s">
+        <v>9</v>
+      </c>
+      <c r="D8" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="E8" s="13" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="13.15" x14ac:dyDescent="0.35">
+      <c r="A9" s="11">
+        <v>46294</v>
+      </c>
+      <c r="B9" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="C9" s="12">
+        <v>1</v>
+      </c>
+      <c r="D9" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="E9" s="9" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="13.15" x14ac:dyDescent="0.35">
+      <c r="A10" s="11">
+        <v>46295</v>
+      </c>
+      <c r="B10" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C10" s="12">
+        <v>1</v>
+      </c>
+      <c r="D10" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="E10" s="9" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="13.15" x14ac:dyDescent="0.35">
+      <c r="A11" s="11">
+        <v>46295</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="C11" s="12">
+        <v>0.5</v>
+      </c>
+      <c r="D11" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="E11" s="9" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="25.5" x14ac:dyDescent="0.35">
+      <c r="A12" s="11">
+        <v>46295</v>
+      </c>
+      <c r="B12" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="C12" s="12">
+        <v>0.5</v>
+      </c>
+      <c r="D12" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="E12" s="9" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="25.5" x14ac:dyDescent="0.35">
+      <c r="A13" s="11">
+        <v>46295</v>
+      </c>
+      <c r="B13" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="C13" s="12">
+        <v>0.5</v>
+      </c>
+      <c r="D13" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="E13" s="9" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="10" t="s">
-        <v>6</v>
-      </c>
-      <c r="B7" s="9"/>
-      <c r="C7" s="9"/>
-      <c r="D7" s="9"/>
-      <c r="E7" s="9"/>
-    </row>
-    <row r="8" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="B8" s="15" t="s">
-        <v>8</v>
-      </c>
-      <c r="C8" s="16" t="s">
-        <v>9</v>
-      </c>
-      <c r="D8" s="15" t="s">
-        <v>10</v>
-      </c>
-      <c r="E8" s="15" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" ht="25.5" x14ac:dyDescent="0.35">
-      <c r="A9" s="13">
-        <v>46294</v>
-      </c>
-      <c r="B9" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="C9" s="14"/>
-      <c r="D9" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="E9" s="11" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" ht="25.5" x14ac:dyDescent="0.35">
-      <c r="A10" s="13">
+    <row r="14" spans="1:5" ht="25.5" x14ac:dyDescent="0.35">
+      <c r="A14" s="11">
         <v>46295</v>
       </c>
-      <c r="B10" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="C10" s="14"/>
-      <c r="D10" s="11" t="s">
-        <v>16</v>
-      </c>
-      <c r="E10" s="11" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" ht="25.5" x14ac:dyDescent="0.35">
-      <c r="A11" s="13">
+      <c r="B14" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="C14" s="12">
+        <v>1.5</v>
+      </c>
+      <c r="D14" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="E14" s="9" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="13.15" x14ac:dyDescent="0.35">
+      <c r="A15" s="11">
         <v>46295</v>
       </c>
-      <c r="B11" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="C11" s="14"/>
-      <c r="D11" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="E11" s="11" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" ht="25.5" x14ac:dyDescent="0.35">
-      <c r="A12" s="13">
+      <c r="B15" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="C15" s="12">
+        <v>0.5</v>
+      </c>
+      <c r="D15" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="E15" s="9" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="25.5" x14ac:dyDescent="0.35">
+      <c r="A16" s="11">
         <v>46295</v>
       </c>
-      <c r="B12" s="12" t="s">
-        <v>21</v>
-      </c>
-      <c r="C12" s="14"/>
-      <c r="D12" s="11" t="s">
-        <v>22</v>
-      </c>
-      <c r="E12" s="11" t="s">
+      <c r="B16" s="10" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" ht="25.5" x14ac:dyDescent="0.35">
-      <c r="A13" s="13">
+      <c r="C16" s="12">
+        <v>1.5</v>
+      </c>
+      <c r="D16" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="E16" s="9" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="26.25" x14ac:dyDescent="0.35">
+      <c r="A17" s="11">
         <v>46295</v>
       </c>
-      <c r="B13" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="C13" s="14"/>
-      <c r="D13" s="11" t="s">
+      <c r="B17" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="E13" s="11" t="s">
+      <c r="C17" s="12">
+        <v>1</v>
+      </c>
+      <c r="D17" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="E17" s="9" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="25.5" x14ac:dyDescent="0.35">
-      <c r="A14" s="13">
+    <row r="18" spans="1:5" ht="26.25" x14ac:dyDescent="0.35">
+      <c r="A18" s="11">
         <v>46295</v>
       </c>
-      <c r="B14" s="12" t="s">
+      <c r="B18" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="C14" s="14"/>
-      <c r="D14" s="11" t="s">
+      <c r="C18" s="12">
+        <v>0.5</v>
+      </c>
+      <c r="D18" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="E18" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="E14" s="11" t="s">
+    </row>
+    <row r="19" spans="1:5" ht="25.5" x14ac:dyDescent="0.35">
+      <c r="A19" s="11">
+        <v>46295</v>
+      </c>
+      <c r="B19" s="10" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="15" spans="1:5" ht="25.5" x14ac:dyDescent="0.35">
-      <c r="A15" s="13">
-        <v>46295</v>
-      </c>
-      <c r="B15" s="12" t="s">
+      <c r="C19" s="12">
+        <v>1.5</v>
+      </c>
+      <c r="D19" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="E19" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="C15" s="14"/>
-      <c r="D15" s="11" t="s">
+    </row>
+    <row r="20" spans="1:5" ht="26.25" x14ac:dyDescent="0.35">
+      <c r="A20" s="11">
+        <v>46296</v>
+      </c>
+      <c r="B20" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="E15" s="11" t="s">
+      <c r="C20" s="12">
+        <v>3</v>
+      </c>
+      <c r="D20" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="E20" s="9" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="16" spans="1:5" ht="38.25" x14ac:dyDescent="0.35">
-      <c r="A16" s="13">
-        <v>46295</v>
-      </c>
-      <c r="B16" s="12" t="s">
+    <row r="21" spans="1:5" ht="25.5" x14ac:dyDescent="0.35">
+      <c r="A21" s="11">
+        <v>46296</v>
+      </c>
+      <c r="B21" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="C16" s="14"/>
-      <c r="D16" s="11" t="s">
+      <c r="C21" s="12">
+        <v>1</v>
+      </c>
+      <c r="D21" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="E21" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="E16" s="11" t="s">
+    </row>
+    <row r="22" spans="1:5" ht="25.5" x14ac:dyDescent="0.35">
+      <c r="A22" s="11">
+        <v>46304</v>
+      </c>
+      <c r="B22" s="10" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="17" spans="1:5" ht="76.5" x14ac:dyDescent="0.35">
-      <c r="A17" s="13">
-        <v>46295</v>
-      </c>
-      <c r="B17" s="12" t="s">
+      <c r="C22" s="12">
+        <v>4</v>
+      </c>
+      <c r="D22" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="E22" s="9" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="25.5" x14ac:dyDescent="0.35">
+      <c r="A23" s="11">
+        <v>46304</v>
+      </c>
+      <c r="B23" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="C17" s="14"/>
-      <c r="D17" s="11" t="s">
+      <c r="C23" s="12">
+        <v>2</v>
+      </c>
+      <c r="D23" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="E23" s="9" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="25.5" x14ac:dyDescent="0.35">
+      <c r="A24" s="11">
+        <v>46304</v>
+      </c>
+      <c r="B24" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="E17" s="11" t="s">
+      <c r="C24" s="12">
+        <v>0.5</v>
+      </c>
+      <c r="D24" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="E24" s="9" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="26.25" x14ac:dyDescent="0.35">
+      <c r="A25" s="11">
+        <v>46304</v>
+      </c>
+      <c r="B25" s="10" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" ht="38.25" x14ac:dyDescent="0.35">
-      <c r="A18" s="13">
-        <v>46295</v>
-      </c>
-      <c r="B18" s="12" t="s">
+      <c r="C25" s="12">
+        <v>1.5</v>
+      </c>
+      <c r="D25" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="E25" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="C18" s="14"/>
-      <c r="D18" s="11" t="s">
+    </row>
+    <row r="26" spans="1:5" ht="26.25" x14ac:dyDescent="0.35">
+      <c r="A26" s="11">
+        <v>46305</v>
+      </c>
+      <c r="B26" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="E18" s="11" t="s">
+      <c r="C26" s="12">
+        <v>2</v>
+      </c>
+      <c r="D26" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="E26" s="9" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="25.5" x14ac:dyDescent="0.35">
+      <c r="A27" s="11">
+        <v>46309</v>
+      </c>
+      <c r="B27" s="10" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" ht="89.25" x14ac:dyDescent="0.35">
-      <c r="A19" s="13">
-        <v>46295</v>
-      </c>
-      <c r="B19" s="12" t="s">
+      <c r="C27" s="12">
+        <v>1</v>
+      </c>
+      <c r="D27" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="E27" s="9" t="s">
         <v>42</v>
-      </c>
-      <c r="C19" s="14"/>
-      <c r="D19" s="11" t="s">
-        <v>43</v>
-      </c>
-      <c r="E19" s="11" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" ht="76.5" x14ac:dyDescent="0.35">
-      <c r="A20" s="13">
-        <v>46296</v>
-      </c>
-      <c r="B20" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="C20" s="14"/>
-      <c r="D20" s="11" t="s">
-        <v>46</v>
-      </c>
-      <c r="E20" s="11" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" ht="76.5" x14ac:dyDescent="0.35">
-      <c r="A21" s="13">
-        <v>46296</v>
-      </c>
-      <c r="B21" s="12" t="s">
-        <v>48</v>
-      </c>
-      <c r="C21" s="14"/>
-      <c r="D21" s="11" t="s">
-        <v>49</v>
-      </c>
-      <c r="E21" s="11" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" ht="114.75" x14ac:dyDescent="0.35">
-      <c r="A22" s="13">
-        <v>46304</v>
-      </c>
-      <c r="B22" s="12" t="s">
-        <v>51</v>
-      </c>
-      <c r="C22" s="14"/>
-      <c r="D22" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="E22" s="11" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" ht="89.25" x14ac:dyDescent="0.35">
-      <c r="A23" s="13">
-        <v>46304</v>
-      </c>
-      <c r="B23" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="C23" s="14"/>
-      <c r="D23" s="11" t="s">
-        <v>55</v>
-      </c>
-      <c r="E23" s="11" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" ht="76.5" x14ac:dyDescent="0.35">
-      <c r="A24" s="13">
-        <v>46304</v>
-      </c>
-      <c r="B24" s="12" t="s">
-        <v>57</v>
-      </c>
-      <c r="C24" s="14"/>
-      <c r="D24" s="11" t="s">
-        <v>58</v>
-      </c>
-      <c r="E24" s="11" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" ht="102" x14ac:dyDescent="0.35">
-      <c r="A25" s="13">
-        <v>46304</v>
-      </c>
-      <c r="B25" s="12" t="s">
-        <v>60</v>
-      </c>
-      <c r="C25" s="14"/>
-      <c r="D25" s="11" t="s">
-        <v>61</v>
-      </c>
-      <c r="E25" s="11" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" ht="102" x14ac:dyDescent="0.35">
-      <c r="A26" s="13">
-        <v>46305</v>
-      </c>
-      <c r="B26" s="12" t="s">
-        <v>63</v>
-      </c>
-      <c r="C26" s="14"/>
-      <c r="D26" s="11" t="s">
-        <v>64</v>
-      </c>
-      <c r="E26" s="11" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" ht="63.75" x14ac:dyDescent="0.35">
-      <c r="A27" s="13">
-        <v>46309</v>
-      </c>
-      <c r="B27" s="12" t="s">
-        <v>65</v>
-      </c>
-      <c r="C27" s="14"/>
-      <c r="D27" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="E27" s="11" t="s">
-        <v>67</v>
       </c>
     </row>
   </sheetData>
@@ -1481,7 +1519,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="26" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A1" s="2" t="s">
-        <v>68</v>
+        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="16.899999999999999" x14ac:dyDescent="0.5">
@@ -1490,427 +1528,427 @@
       </c>
     </row>
     <row r="3" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="10" t="s">
-        <v>69</v>
-      </c>
-      <c r="B3" s="9"/>
-      <c r="C3" s="9"/>
-      <c r="D3" s="9"/>
-      <c r="E3" s="9"/>
+      <c r="A3" s="31" t="s">
+        <v>44</v>
+      </c>
+      <c r="B3" s="32"/>
+      <c r="C3" s="32"/>
+      <c r="D3" s="32"/>
+      <c r="E3" s="32"/>
     </row>
     <row r="5" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="18" t="s">
-        <v>70</v>
-      </c>
-      <c r="B5" s="18" t="s">
-        <v>71</v>
-      </c>
-      <c r="C5" s="18" t="s">
-        <v>72</v>
-      </c>
-      <c r="D5" s="18" t="s">
+      <c r="A5" s="16" t="s">
+        <v>45</v>
+      </c>
+      <c r="B5" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="C5" s="16" t="s">
+        <v>47</v>
+      </c>
+      <c r="D5" s="16" t="s">
         <v>9</v>
       </c>
-      <c r="E5" s="18" t="s">
-        <v>73</v>
+      <c r="E5" s="16" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A6" s="19">
+      <c r="A6" s="17">
         <v>46293</v>
       </c>
-      <c r="B6" s="20">
-        <f>A6+6</f>
+      <c r="B6" s="18">
+        <f t="shared" ref="B6:B21" si="0">A6+6</f>
         <v>46299</v>
       </c>
-      <c r="C6" s="21">
+      <c r="C6" s="19">
         <f>COUNTIFS(Registro[Data],"&gt;="&amp;A6,Registro[Data],"&lt;="&amp;B6)</f>
         <v>13</v>
       </c>
-      <c r="D6" s="22">
+      <c r="D6" s="20">
         <f>SUMIFS(Registro[Ore],Registro[Data],"&gt;="&amp;A6,Registro[Data],"&lt;="&amp;B6)</f>
-        <v>0</v>
-      </c>
-      <c r="E6" s="22">
+        <v>14</v>
+      </c>
+      <c r="E6" s="20">
         <f>SUM(D$6:D6)</f>
-        <v>0</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A7" s="23">
-        <f>A6+7</f>
+      <c r="A7" s="21">
+        <f t="shared" ref="A7:A21" si="1">A6+7</f>
         <v>46300</v>
       </c>
-      <c r="B7" s="23">
-        <f>A7+6</f>
+      <c r="B7" s="21">
+        <f t="shared" si="0"/>
         <v>46306</v>
       </c>
-      <c r="C7" s="24">
+      <c r="C7" s="22">
         <f>COUNTIFS(Registro[Data],"&gt;="&amp;A7,Registro[Data],"&lt;="&amp;B7)</f>
         <v>5</v>
       </c>
-      <c r="D7" s="25">
+      <c r="D7" s="23">
         <f>SUMIFS(Registro[Ore],Registro[Data],"&gt;="&amp;A7,Registro[Data],"&lt;="&amp;B7)</f>
-        <v>0</v>
-      </c>
-      <c r="E7" s="25">
+        <v>10</v>
+      </c>
+      <c r="E7" s="23">
         <f>SUM(D$6:D7)</f>
-        <v>0</v>
+        <v>24</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A8" s="20">
-        <f>A7+7</f>
+      <c r="A8" s="18">
+        <f t="shared" si="1"/>
         <v>46307</v>
       </c>
-      <c r="B8" s="20">
-        <f>A8+6</f>
+      <c r="B8" s="18">
+        <f t="shared" si="0"/>
         <v>46313</v>
       </c>
-      <c r="C8" s="21">
+      <c r="C8" s="19">
         <f>COUNTIFS(Registro[Data],"&gt;="&amp;A8,Registro[Data],"&lt;="&amp;B8)</f>
         <v>1</v>
       </c>
-      <c r="D8" s="22">
+      <c r="D8" s="20">
         <f>SUMIFS(Registro[Ore],Registro[Data],"&gt;="&amp;A8,Registro[Data],"&lt;="&amp;B8)</f>
-        <v>0</v>
-      </c>
-      <c r="E8" s="22">
+        <v>1</v>
+      </c>
+      <c r="E8" s="20">
         <f>SUM(D$6:D8)</f>
-        <v>0</v>
+        <v>25</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A9" s="23">
-        <f>A8+7</f>
+      <c r="A9" s="21">
+        <f t="shared" si="1"/>
         <v>46314</v>
       </c>
-      <c r="B9" s="23">
-        <f>A9+6</f>
+      <c r="B9" s="21">
+        <f t="shared" si="0"/>
         <v>46320</v>
       </c>
-      <c r="C9" s="24">
+      <c r="C9" s="22">
         <f>COUNTIFS(Registro[Data],"&gt;="&amp;A9,Registro[Data],"&lt;="&amp;B9)</f>
         <v>0</v>
       </c>
-      <c r="D9" s="25">
+      <c r="D9" s="23">
         <f>SUMIFS(Registro[Ore],Registro[Data],"&gt;="&amp;A9,Registro[Data],"&lt;="&amp;B9)</f>
         <v>0</v>
       </c>
-      <c r="E9" s="25">
+      <c r="E9" s="23">
         <f>SUM(D$6:D9)</f>
-        <v>0</v>
+        <v>25</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A10" s="20">
-        <f>A9+7</f>
+      <c r="A10" s="18">
+        <f t="shared" si="1"/>
         <v>46321</v>
       </c>
-      <c r="B10" s="20">
-        <f>A10+6</f>
+      <c r="B10" s="18">
+        <f t="shared" si="0"/>
         <v>46327</v>
       </c>
-      <c r="C10" s="21">
+      <c r="C10" s="19">
         <f>COUNTIFS(Registro[Data],"&gt;="&amp;A10,Registro[Data],"&lt;="&amp;B10)</f>
         <v>0</v>
       </c>
-      <c r="D10" s="22">
+      <c r="D10" s="20">
         <f>SUMIFS(Registro[Ore],Registro[Data],"&gt;="&amp;A10,Registro[Data],"&lt;="&amp;B10)</f>
         <v>0</v>
       </c>
-      <c r="E10" s="22">
+      <c r="E10" s="20">
         <f>SUM(D$6:D10)</f>
-        <v>0</v>
+        <v>25</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A11" s="23">
-        <f>A10+7</f>
+      <c r="A11" s="21">
+        <f t="shared" si="1"/>
         <v>46328</v>
       </c>
-      <c r="B11" s="23">
-        <f>A11+6</f>
+      <c r="B11" s="21">
+        <f t="shared" si="0"/>
         <v>46334</v>
       </c>
-      <c r="C11" s="24">
+      <c r="C11" s="22">
         <f>COUNTIFS(Registro[Data],"&gt;="&amp;A11,Registro[Data],"&lt;="&amp;B11)</f>
         <v>0</v>
       </c>
-      <c r="D11" s="25">
+      <c r="D11" s="23">
         <f>SUMIFS(Registro[Ore],Registro[Data],"&gt;="&amp;A11,Registro[Data],"&lt;="&amp;B11)</f>
         <v>0</v>
       </c>
-      <c r="E11" s="25">
+      <c r="E11" s="23">
         <f>SUM(D$6:D11)</f>
-        <v>0</v>
+        <v>25</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A12" s="20">
-        <f>A11+7</f>
+      <c r="A12" s="18">
+        <f t="shared" si="1"/>
         <v>46335</v>
       </c>
-      <c r="B12" s="20">
-        <f>A12+6</f>
+      <c r="B12" s="18">
+        <f t="shared" si="0"/>
         <v>46341</v>
       </c>
-      <c r="C12" s="21">
+      <c r="C12" s="19">
         <f>COUNTIFS(Registro[Data],"&gt;="&amp;A12,Registro[Data],"&lt;="&amp;B12)</f>
         <v>0</v>
       </c>
-      <c r="D12" s="22">
+      <c r="D12" s="20">
         <f>SUMIFS(Registro[Ore],Registro[Data],"&gt;="&amp;A12,Registro[Data],"&lt;="&amp;B12)</f>
         <v>0</v>
       </c>
-      <c r="E12" s="22">
+      <c r="E12" s="20">
         <f>SUM(D$6:D12)</f>
-        <v>0</v>
+        <v>25</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A13" s="23">
-        <f>A12+7</f>
+      <c r="A13" s="21">
+        <f t="shared" si="1"/>
         <v>46342</v>
       </c>
-      <c r="B13" s="23">
-        <f>A13+6</f>
+      <c r="B13" s="21">
+        <f t="shared" si="0"/>
         <v>46348</v>
       </c>
-      <c r="C13" s="24">
+      <c r="C13" s="22">
         <f>COUNTIFS(Registro[Data],"&gt;="&amp;A13,Registro[Data],"&lt;="&amp;B13)</f>
         <v>0</v>
       </c>
-      <c r="D13" s="25">
+      <c r="D13" s="23">
         <f>SUMIFS(Registro[Ore],Registro[Data],"&gt;="&amp;A13,Registro[Data],"&lt;="&amp;B13)</f>
         <v>0</v>
       </c>
-      <c r="E13" s="25">
+      <c r="E13" s="23">
         <f>SUM(D$6:D13)</f>
-        <v>0</v>
+        <v>25</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A14" s="20">
-        <f>A13+7</f>
+      <c r="A14" s="18">
+        <f t="shared" si="1"/>
         <v>46349</v>
       </c>
-      <c r="B14" s="20">
-        <f>A14+6</f>
+      <c r="B14" s="18">
+        <f t="shared" si="0"/>
         <v>46355</v>
       </c>
-      <c r="C14" s="21">
+      <c r="C14" s="19">
         <f>COUNTIFS(Registro[Data],"&gt;="&amp;A14,Registro[Data],"&lt;="&amp;B14)</f>
         <v>0</v>
       </c>
-      <c r="D14" s="22">
+      <c r="D14" s="20">
         <f>SUMIFS(Registro[Ore],Registro[Data],"&gt;="&amp;A14,Registro[Data],"&lt;="&amp;B14)</f>
         <v>0</v>
       </c>
-      <c r="E14" s="22">
+      <c r="E14" s="20">
         <f>SUM(D$6:D14)</f>
-        <v>0</v>
+        <v>25</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A15" s="23">
-        <f>A14+7</f>
+      <c r="A15" s="21">
+        <f t="shared" si="1"/>
         <v>46356</v>
       </c>
-      <c r="B15" s="23">
-        <f>A15+6</f>
+      <c r="B15" s="21">
+        <f t="shared" si="0"/>
         <v>46362</v>
       </c>
-      <c r="C15" s="24">
+      <c r="C15" s="22">
         <f>COUNTIFS(Registro[Data],"&gt;="&amp;A15,Registro[Data],"&lt;="&amp;B15)</f>
         <v>0</v>
       </c>
-      <c r="D15" s="25">
+      <c r="D15" s="23">
         <f>SUMIFS(Registro[Ore],Registro[Data],"&gt;="&amp;A15,Registro[Data],"&lt;="&amp;B15)</f>
         <v>0</v>
       </c>
-      <c r="E15" s="25">
+      <c r="E15" s="23">
         <f>SUM(D$6:D15)</f>
-        <v>0</v>
+        <v>25</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A16" s="20">
-        <f>A15+7</f>
+      <c r="A16" s="18">
+        <f t="shared" si="1"/>
         <v>46363</v>
       </c>
-      <c r="B16" s="20">
-        <f>A16+6</f>
+      <c r="B16" s="18">
+        <f t="shared" si="0"/>
         <v>46369</v>
       </c>
-      <c r="C16" s="21">
+      <c r="C16" s="19">
         <f>COUNTIFS(Registro[Data],"&gt;="&amp;A16,Registro[Data],"&lt;="&amp;B16)</f>
         <v>0</v>
       </c>
-      <c r="D16" s="22">
+      <c r="D16" s="20">
         <f>SUMIFS(Registro[Ore],Registro[Data],"&gt;="&amp;A16,Registro[Data],"&lt;="&amp;B16)</f>
         <v>0</v>
       </c>
-      <c r="E16" s="22">
+      <c r="E16" s="20">
         <f>SUM(D$6:D16)</f>
-        <v>0</v>
+        <v>25</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A17" s="23">
-        <f>A16+7</f>
+      <c r="A17" s="21">
+        <f t="shared" si="1"/>
         <v>46370</v>
       </c>
-      <c r="B17" s="23">
-        <f>A17+6</f>
+      <c r="B17" s="21">
+        <f t="shared" si="0"/>
         <v>46376</v>
       </c>
-      <c r="C17" s="24">
+      <c r="C17" s="22">
         <f>COUNTIFS(Registro[Data],"&gt;="&amp;A17,Registro[Data],"&lt;="&amp;B17)</f>
         <v>0</v>
       </c>
-      <c r="D17" s="25">
+      <c r="D17" s="23">
         <f>SUMIFS(Registro[Ore],Registro[Data],"&gt;="&amp;A17,Registro[Data],"&lt;="&amp;B17)</f>
         <v>0</v>
       </c>
-      <c r="E17" s="25">
+      <c r="E17" s="23">
         <f>SUM(D$6:D17)</f>
-        <v>0</v>
+        <v>25</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A18" s="20">
-        <f>A17+7</f>
+      <c r="A18" s="18">
+        <f t="shared" si="1"/>
         <v>46377</v>
       </c>
-      <c r="B18" s="20">
-        <f>A18+6</f>
+      <c r="B18" s="18">
+        <f t="shared" si="0"/>
         <v>46383</v>
       </c>
-      <c r="C18" s="21">
+      <c r="C18" s="19">
         <f>COUNTIFS(Registro[Data],"&gt;="&amp;A18,Registro[Data],"&lt;="&amp;B18)</f>
         <v>0</v>
       </c>
-      <c r="D18" s="22">
+      <c r="D18" s="20">
         <f>SUMIFS(Registro[Ore],Registro[Data],"&gt;="&amp;A18,Registro[Data],"&lt;="&amp;B18)</f>
         <v>0</v>
       </c>
-      <c r="E18" s="22">
+      <c r="E18" s="20">
         <f>SUM(D$6:D18)</f>
-        <v>0</v>
+        <v>25</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A19" s="23">
-        <f>A18+7</f>
+      <c r="A19" s="21">
+        <f t="shared" si="1"/>
         <v>46384</v>
       </c>
-      <c r="B19" s="23">
-        <f>A19+6</f>
+      <c r="B19" s="21">
+        <f t="shared" si="0"/>
         <v>46390</v>
       </c>
-      <c r="C19" s="24">
+      <c r="C19" s="22">
         <f>COUNTIFS(Registro[Data],"&gt;="&amp;A19,Registro[Data],"&lt;="&amp;B19)</f>
         <v>0</v>
       </c>
-      <c r="D19" s="25">
+      <c r="D19" s="23">
         <f>SUMIFS(Registro[Ore],Registro[Data],"&gt;="&amp;A19,Registro[Data],"&lt;="&amp;B19)</f>
         <v>0</v>
       </c>
-      <c r="E19" s="25">
+      <c r="E19" s="23">
         <f>SUM(D$6:D19)</f>
-        <v>0</v>
+        <v>25</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A20" s="20">
-        <f>A19+7</f>
+      <c r="A20" s="18">
+        <f t="shared" si="1"/>
         <v>46391</v>
       </c>
-      <c r="B20" s="20">
-        <f>A20+6</f>
+      <c r="B20" s="18">
+        <f t="shared" si="0"/>
         <v>46397</v>
       </c>
-      <c r="C20" s="21">
+      <c r="C20" s="19">
         <f>COUNTIFS(Registro[Data],"&gt;="&amp;A20,Registro[Data],"&lt;="&amp;B20)</f>
         <v>0</v>
       </c>
-      <c r="D20" s="22">
+      <c r="D20" s="20">
         <f>SUMIFS(Registro[Ore],Registro[Data],"&gt;="&amp;A20,Registro[Data],"&lt;="&amp;B20)</f>
         <v>0</v>
       </c>
-      <c r="E20" s="22">
+      <c r="E20" s="20">
         <f>SUM(D$6:D20)</f>
-        <v>0</v>
+        <v>25</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A21" s="26">
-        <f>A20+7</f>
+      <c r="A21" s="24">
+        <f t="shared" si="1"/>
         <v>46398</v>
       </c>
-      <c r="B21" s="26">
-        <f>A21+6</f>
+      <c r="B21" s="24">
+        <f t="shared" si="0"/>
         <v>46404</v>
       </c>
-      <c r="C21" s="27">
+      <c r="C21" s="25">
         <f>COUNTIFS(Registro[Data],"&gt;="&amp;A21,Registro[Data],"&lt;="&amp;B21)</f>
         <v>0</v>
       </c>
-      <c r="D21" s="28">
+      <c r="D21" s="26">
         <f>SUMIFS(Registro[Ore],Registro[Data],"&gt;="&amp;A21,Registro[Data],"&lt;="&amp;B21)</f>
         <v>0</v>
       </c>
-      <c r="E21" s="28">
+      <c r="E21" s="26">
         <f>SUM(D$6:D21)</f>
-        <v>0</v>
+        <v>25</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="13.15" x14ac:dyDescent="0.4">
-      <c r="A22" s="29" t="s">
-        <v>74</v>
-      </c>
-      <c r="B22" s="30"/>
-      <c r="C22" s="31">
+      <c r="A22" s="27" t="s">
+        <v>49</v>
+      </c>
+      <c r="B22" s="28"/>
+      <c r="C22" s="29">
         <f>SUM(C6:C21)</f>
         <v>19</v>
       </c>
-      <c r="D22" s="32">
+      <c r="D22" s="30">
         <f>SUM(D6:D21)</f>
-        <v>0</v>
-      </c>
-      <c r="E22" s="30"/>
+        <v>25</v>
+      </c>
+      <c r="E22" s="28"/>
     </row>
     <row r="24" spans="1:5" ht="13.15" x14ac:dyDescent="0.4">
       <c r="A24" s="6" t="s">
-        <v>75</v>
+        <v>50</v>
       </c>
       <c r="B24" s="6"/>
       <c r="C24" s="6"/>
-      <c r="D24" s="17">
+      <c r="D24" s="15">
         <f>SUM(Registro[Ore])</f>
-        <v>0</v>
+        <v>25</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="13.15" x14ac:dyDescent="0.4">
       <c r="A25" s="6" t="s">
-        <v>76</v>
+        <v>51</v>
       </c>
       <c r="B25" s="6"/>
       <c r="C25" s="6"/>
-      <c r="D25" s="17">
+      <c r="D25" s="15">
         <f>D24-D22</f>
         <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="10" t="s">
-        <v>77</v>
-      </c>
-      <c r="B26" s="9"/>
-      <c r="C26" s="9"/>
-      <c r="D26" s="9"/>
-      <c r="E26" s="9"/>
+      <c r="A26" s="31" t="s">
+        <v>52</v>
+      </c>
+      <c r="B26" s="32"/>
+      <c r="C26" s="32"/>
+      <c r="D26" s="32"/>
+      <c r="E26" s="32"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
Elenco dei compiti in un unico Excel
Cose mancanti e checklist GDPR passano in docs/compiti.xlsx: una riga per
voce, con assegnatario, stato (da fare rosso, in corso giallo, fatto verde),
data di fine, note e un riepilogo automatico. Rimossi i due file Markdown e
aggiornati i collegamenti nei README. Voce nel libretto di Manuel.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/libretti/manuel-bulla.xlsx
+++ b/docs/libretti/manuel-bulla.xlsx
@@ -734,8 +734,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F7E690B7-EC62-4BC2-A27A-E592475A3F24}" name="Registro" displayName="Registro" ref="A8:E27" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
-  <autoFilter ref="A8:E27" xr:uid="{F7E690B7-EC62-4BC2-A27A-E592475A3F24}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F7E690B7-EC62-4BC2-A27A-E592475A3F24}" name="Registro" displayName="Registro" ref="A8:E28" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
+  <autoFilter ref="A8:E28" xr:uid="{F7E690B7-EC62-4BC2-A27A-E592475A3F24}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
@@ -1471,21 +1471,44 @@
         <v>42</v>
       </c>
     </row>
+    <row r="28" spans="1:5" ht="25.5" x14ac:dyDescent="0.35">
+      <c r="A28" s="11">
+        <v>46309</v>
+      </c>
+      <c r="B28" s="10" t="inlineStr">
+        <is>
+          <t>Elenco dei compiti in Excel</t>
+        </is>
+      </c>
+      <c r="C28" s="12">
+        <v>1</v>
+      </c>
+      <c r="D28" s="9" t="inlineStr">
+        <is>
+          <t>Uniti i documenti sulle cose mancanti e sulla checklist GDPR in un solo foglio Excel, con assegnatario e stato (da fare rosso, in corso giallo, fatto verde); rimossi i due file Markdown.</t>
+        </is>
+      </c>
+      <c r="E28" s="9" t="inlineStr">
+        <is>
+          <t>docs/compiti.xlsx</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A7:E7"/>
   </mergeCells>
-  <conditionalFormatting sqref="C9:C27">
+  <conditionalFormatting sqref="C9:C28">
     <cfRule type="expression" dxfId="1" priority="1" stopIfTrue="1">
       <formula>($B9&lt;&gt;"")*($C9="")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Data non valida" error="Scrivi la data come gg/mm/aaaa, per esempio 14/10/2026." sqref="A9:A27" xr:uid="{D26B2BD8-0AFD-48FB-BBA1-B07F75408464}">
+    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Data non valida" error="Scrivi la data come gg/mm/aaaa, per esempio 14/10/2026." sqref="A9:A28" xr:uid="{D26B2BD8-0AFD-48FB-BBA1-B07F75408464}">
       <formula1>46023</formula1>
       <formula2>47483</formula2>
     </dataValidation>
-    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Ore non valide" error="Scrivi le ore come numero tra 0 e 24 (1,5 = un'ora e mezza)." promptTitle="Ore dedicate" prompt="Numero di ore, anche decimale: 1,5 = un'ora e mezza." sqref="C9:C27" xr:uid="{04EB0103-1D9C-4DFC-8906-92996DF6DE7A}">
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Ore non valide" error="Scrivi le ore come numero tra 0 e 24 (1,5 = un'ora e mezza)." promptTitle="Ore dedicate" prompt="Numero di ore, anche decimale: 1,5 = un'ora e mezza." sqref="C9:C28" xr:uid="{04EB0103-1D9C-4DFC-8906-92996DF6DE7A}">
       <formula1>0</formula1>
       <formula2>24</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
Sfondo della mappa con MapTiler
Stile "dataviz-light" (senza negozi e bar) al posto dei tile standard di OpenStreetMap, proposto da Marco.
La chiave sta in VITE_MAPTILER_KEY (frontend/.env.local, ignorato da Git; build Docker con ARG);
senza chiave si ripiega su OpenStreetMap. Aggiornati CSP, informativa e crediti in italiano, inglese e tedesco.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/libretti/manuel-bulla.xlsx
+++ b/docs/libretti/manuel-bulla.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bulla\Documents\Ing-software-v1\docs\libretti\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{013AFA0A-E8BA-4C2C-BB7E-2AD1444DD5A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C072062B-DEEC-46F7-8B68-E8D8ED11DC04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{EB300ADB-58B5-479D-B51B-E912DFEACD78}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="87">
   <si>
     <t>Libretto delle attività</t>
   </si>
@@ -295,6 +295,15 @@
   </si>
   <si>
     <t>versione-corrente/frontend/src/i18n/de.js, versione-corrente/backend/src/db/dati/004-traduzioni-tedesche/</t>
+  </si>
+  <si>
+    <t>Sfondo mappa MapTiler</t>
+  </si>
+  <si>
+    <t>Sostituito lo sfondo OpenStreetMap con lo stile MapTiler "dataviz-light" (senza negozi e bar), proposto da Marco. Chiave in .env.local, ripiego su OSM senza chiave, testi in tre lingue.</t>
+  </si>
+  <si>
+    <t>versione-corrente/frontend/src/lib/sfondo.js, MappaLeaflet.jsx, Copertina.jsx, .env.esempio</t>
   </si>
 </sst>
 </file>
@@ -752,8 +761,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F7E690B7-EC62-4BC2-A27A-E592475A3F24}" name="Registro" displayName="Registro" ref="A8:E29" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
-  <autoFilter ref="A8:E29" xr:uid="{F7E690B7-EC62-4BC2-A27A-E592475A3F24}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F7E690B7-EC62-4BC2-A27A-E592475A3F24}" name="Registro" displayName="Registro" ref="A8:E30" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
+  <autoFilter ref="A8:E30" xr:uid="{F7E690B7-EC62-4BC2-A27A-E592475A3F24}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
@@ -1091,7 +1100,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E30"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.59765625" style="1" customWidth="1"/>
@@ -1128,7 +1137,7 @@
       </c>
       <c r="C5" s="7">
         <f>SUM(Registro[Ore])</f>
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="13.15" x14ac:dyDescent="0.4">
@@ -1523,21 +1532,38 @@
         <v>83</v>
       </c>
     </row>
+    <row r="30" spans="1:5" ht="38.25" x14ac:dyDescent="0.35">
+      <c r="A30" s="11">
+        <v>46309</v>
+      </c>
+      <c r="B30" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="C30" s="12">
+        <v>1</v>
+      </c>
+      <c r="D30" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="E30" s="9" t="s">
+        <v>86</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A7:E7"/>
   </mergeCells>
-  <conditionalFormatting sqref="C9:C29">
+  <conditionalFormatting sqref="C9:C30">
     <cfRule type="expression" dxfId="1" priority="1" stopIfTrue="1">
       <formula>($B9&lt;&gt;"")*($C9="")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Data non valida" error="Scrivi la data come gg/mm/aaaa, per esempio 14/10/2026." sqref="A9:A29" xr:uid="{D26B2BD8-0AFD-48FB-BBA1-B07F75408464}">
+    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Data non valida" error="Scrivi la data come gg/mm/aaaa, per esempio 14/10/2026." sqref="A9:A30" xr:uid="{D26B2BD8-0AFD-48FB-BBA1-B07F75408464}">
       <formula1>46023</formula1>
       <formula2>47483</formula2>
     </dataValidation>
-    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Ore non valide" error="Scrivi le ore come numero tra 0 e 24 (1,5 = un'ora e mezza)." promptTitle="Ore dedicate" prompt="Numero di ore, anche decimale: 1,5 = un'ora e mezza." sqref="C9:C29" xr:uid="{04EB0103-1D9C-4DFC-8906-92996DF6DE7A}">
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Ore non valide" error="Scrivi le ore come numero tra 0 e 24 (1,5 = un'ora e mezza)." promptTitle="Ore dedicate" prompt="Numero di ore, anche decimale: 1,5 = un'ora e mezza." sqref="C9:C30" xr:uid="{04EB0103-1D9C-4DFC-8906-92996DF6DE7A}">
       <formula1>0</formula1>
       <formula2>24</formula2>
     </dataValidation>
@@ -1659,15 +1685,15 @@
       </c>
       <c r="C8" s="19">
         <f>COUNTIFS(Registro[Data],"&gt;="&amp;A8,Registro[Data],"&lt;="&amp;B8)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D8" s="20">
         <f>SUMIFS(Registro[Ore],Registro[Data],"&gt;="&amp;A8,Registro[Data],"&lt;="&amp;B8)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E8" s="20">
         <f>SUM(D$6:D8)</f>
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
@@ -1689,7 +1715,7 @@
       </c>
       <c r="E9" s="23">
         <f>SUM(D$6:D9)</f>
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
@@ -1711,7 +1737,7 @@
       </c>
       <c r="E10" s="20">
         <f>SUM(D$6:D10)</f>
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.35">
@@ -1733,7 +1759,7 @@
       </c>
       <c r="E11" s="23">
         <f>SUM(D$6:D11)</f>
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.35">
@@ -1755,7 +1781,7 @@
       </c>
       <c r="E12" s="20">
         <f>SUM(D$6:D12)</f>
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
@@ -1777,7 +1803,7 @@
       </c>
       <c r="E13" s="23">
         <f>SUM(D$6:D13)</f>
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
@@ -1799,7 +1825,7 @@
       </c>
       <c r="E14" s="20">
         <f>SUM(D$6:D14)</f>
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.35">
@@ -1821,7 +1847,7 @@
       </c>
       <c r="E15" s="23">
         <f>SUM(D$6:D15)</f>
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.35">
@@ -1843,7 +1869,7 @@
       </c>
       <c r="E16" s="20">
         <f>SUM(D$6:D16)</f>
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.35">
@@ -1865,7 +1891,7 @@
       </c>
       <c r="E17" s="23">
         <f>SUM(D$6:D17)</f>
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.35">
@@ -1887,7 +1913,7 @@
       </c>
       <c r="E18" s="20">
         <f>SUM(D$6:D18)</f>
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.35">
@@ -1909,7 +1935,7 @@
       </c>
       <c r="E19" s="23">
         <f>SUM(D$6:D19)</f>
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.35">
@@ -1931,7 +1957,7 @@
       </c>
       <c r="E20" s="20">
         <f>SUM(D$6:D20)</f>
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.35">
@@ -1953,7 +1979,7 @@
       </c>
       <c r="E21" s="26">
         <f>SUM(D$6:D21)</f>
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="13.15" x14ac:dyDescent="0.4">
@@ -1963,11 +1989,11 @@
       <c r="B22" s="28"/>
       <c r="C22" s="29">
         <f>SUM(C6:C21)</f>
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D22" s="30">
         <f>SUM(D6:D21)</f>
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E22" s="28"/>
     </row>
@@ -1979,7 +2005,7 @@
       <c r="C24" s="6"/>
       <c r="D24" s="15">
         <f>SUM(Registro[Ore])</f>
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="13.15" x14ac:dyDescent="0.4">

</xml_diff>

<commit_message>
Pulsante per la vista satellitare sulla mappa
Un pulsante in basso a sinistra passa dalla mappa normale al satellite di MapTiler e ricorda la scelta.
Presente sulle mappe interattive, non nel gioco "Dov'era?". Testi in italiano, inglese e tedesco.
Aggiunte le voci nei libretti di Manuel e di Pietro.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/libretti/manuel-bulla.xlsx
+++ b/docs/libretti/manuel-bulla.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bulla\Documents\Ing-software-v1\docs\libretti\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C072062B-DEEC-46F7-8B68-E8D8ED11DC04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C69A8E71-3EB6-4B3F-B117-231ACE64114D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{EB300ADB-58B5-479D-B51B-E912DFEACD78}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="90">
   <si>
     <t>Libretto delle attività</t>
   </si>
@@ -304,6 +304,15 @@
   </si>
   <si>
     <t>versione-corrente/frontend/src/lib/sfondo.js, MappaLeaflet.jsx, Copertina.jsx, .env.esempio</t>
+  </si>
+  <si>
+    <t>Pulsante vista satellitare</t>
+  </si>
+  <si>
+    <t>Aggiunto alla mappa un pulsante per passare dalla vista normale a quella satellitare (MapTiler), ricordando la scelta; assente nel gioco "Dov'era?".</t>
+  </si>
+  <si>
+    <t>versione-corrente/frontend/src/components/MappaLeaflet.jsx, lib/sfondo.js, stile.css, i18n</t>
   </si>
 </sst>
 </file>
@@ -761,8 +770,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F7E690B7-EC62-4BC2-A27A-E592475A3F24}" name="Registro" displayName="Registro" ref="A8:E30" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
-  <autoFilter ref="A8:E30" xr:uid="{F7E690B7-EC62-4BC2-A27A-E592475A3F24}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F7E690B7-EC62-4BC2-A27A-E592475A3F24}" name="Registro" displayName="Registro" ref="A8:E31" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
+  <autoFilter ref="A8:E31" xr:uid="{F7E690B7-EC62-4BC2-A27A-E592475A3F24}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
@@ -1100,7 +1109,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.59765625" style="1" customWidth="1"/>
@@ -1137,7 +1146,7 @@
       </c>
       <c r="C5" s="7">
         <f>SUM(Registro[Ore])</f>
-        <v>33</v>
+        <v>34.5</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="13.15" x14ac:dyDescent="0.4">
@@ -1549,21 +1558,38 @@
         <v>86</v>
       </c>
     </row>
+    <row r="31" spans="1:5" ht="38.25" x14ac:dyDescent="0.35">
+      <c r="A31" s="11">
+        <v>46310</v>
+      </c>
+      <c r="B31" s="10" t="s">
+        <v>87</v>
+      </c>
+      <c r="C31" s="12">
+        <v>1.5</v>
+      </c>
+      <c r="D31" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="E31" s="9" t="s">
+        <v>89</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A7:E7"/>
   </mergeCells>
-  <conditionalFormatting sqref="C9:C30">
+  <conditionalFormatting sqref="C9:C31">
     <cfRule type="expression" dxfId="1" priority="1" stopIfTrue="1">
       <formula>($B9&lt;&gt;"")*($C9="")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Data non valida" error="Scrivi la data come gg/mm/aaaa, per esempio 14/10/2026." sqref="A9:A30" xr:uid="{D26B2BD8-0AFD-48FB-BBA1-B07F75408464}">
+    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Data non valida" error="Scrivi la data come gg/mm/aaaa, per esempio 14/10/2026." sqref="A9:A31" xr:uid="{D26B2BD8-0AFD-48FB-BBA1-B07F75408464}">
       <formula1>46023</formula1>
       <formula2>47483</formula2>
     </dataValidation>
-    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Ore non valide" error="Scrivi le ore come numero tra 0 e 24 (1,5 = un'ora e mezza)." promptTitle="Ore dedicate" prompt="Numero di ore, anche decimale: 1,5 = un'ora e mezza." sqref="C9:C30" xr:uid="{04EB0103-1D9C-4DFC-8906-92996DF6DE7A}">
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Ore non valide" error="Scrivi le ore come numero tra 0 e 24 (1,5 = un'ora e mezza)." promptTitle="Ore dedicate" prompt="Numero di ore, anche decimale: 1,5 = un'ora e mezza." sqref="C9:C31" xr:uid="{04EB0103-1D9C-4DFC-8906-92996DF6DE7A}">
       <formula1>0</formula1>
       <formula2>24</formula2>
     </dataValidation>
@@ -1685,15 +1711,15 @@
       </c>
       <c r="C8" s="19">
         <f>COUNTIFS(Registro[Data],"&gt;="&amp;A8,Registro[Data],"&lt;="&amp;B8)</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D8" s="20">
         <f>SUMIFS(Registro[Ore],Registro[Data],"&gt;="&amp;A8,Registro[Data],"&lt;="&amp;B8)</f>
-        <v>7</v>
+        <v>8.5</v>
       </c>
       <c r="E8" s="20">
         <f>SUM(D$6:D8)</f>
-        <v>33</v>
+        <v>34.5</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
@@ -1715,7 +1741,7 @@
       </c>
       <c r="E9" s="23">
         <f>SUM(D$6:D9)</f>
-        <v>33</v>
+        <v>34.5</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
@@ -1737,7 +1763,7 @@
       </c>
       <c r="E10" s="20">
         <f>SUM(D$6:D10)</f>
-        <v>33</v>
+        <v>34.5</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.35">
@@ -1759,7 +1785,7 @@
       </c>
       <c r="E11" s="23">
         <f>SUM(D$6:D11)</f>
-        <v>33</v>
+        <v>34.5</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.35">
@@ -1781,7 +1807,7 @@
       </c>
       <c r="E12" s="20">
         <f>SUM(D$6:D12)</f>
-        <v>33</v>
+        <v>34.5</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
@@ -1803,7 +1829,7 @@
       </c>
       <c r="E13" s="23">
         <f>SUM(D$6:D13)</f>
-        <v>33</v>
+        <v>34.5</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
@@ -1825,7 +1851,7 @@
       </c>
       <c r="E14" s="20">
         <f>SUM(D$6:D14)</f>
-        <v>33</v>
+        <v>34.5</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.35">
@@ -1847,7 +1873,7 @@
       </c>
       <c r="E15" s="23">
         <f>SUM(D$6:D15)</f>
-        <v>33</v>
+        <v>34.5</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.35">
@@ -1869,7 +1895,7 @@
       </c>
       <c r="E16" s="20">
         <f>SUM(D$6:D16)</f>
-        <v>33</v>
+        <v>34.5</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.35">
@@ -1891,7 +1917,7 @@
       </c>
       <c r="E17" s="23">
         <f>SUM(D$6:D17)</f>
-        <v>33</v>
+        <v>34.5</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.35">
@@ -1913,7 +1939,7 @@
       </c>
       <c r="E18" s="20">
         <f>SUM(D$6:D18)</f>
-        <v>33</v>
+        <v>34.5</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.35">
@@ -1935,7 +1961,7 @@
       </c>
       <c r="E19" s="23">
         <f>SUM(D$6:D19)</f>
-        <v>33</v>
+        <v>34.5</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.35">
@@ -1957,7 +1983,7 @@
       </c>
       <c r="E20" s="20">
         <f>SUM(D$6:D20)</f>
-        <v>33</v>
+        <v>34.5</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.35">
@@ -1979,7 +2005,7 @@
       </c>
       <c r="E21" s="26">
         <f>SUM(D$6:D21)</f>
-        <v>33</v>
+        <v>34.5</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="13.15" x14ac:dyDescent="0.4">
@@ -1989,11 +2015,11 @@
       <c r="B22" s="28"/>
       <c r="C22" s="29">
         <f>SUM(C6:C21)</f>
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D22" s="30">
         <f>SUM(D6:D21)</f>
-        <v>33</v>
+        <v>34.5</v>
       </c>
       <c r="E22" s="28"/>
     </row>
@@ -2005,7 +2031,7 @@
       <c r="C24" s="6"/>
       <c r="D24" s="15">
         <f>SUM(Registro[Ore])</f>
-        <v>33</v>
+        <v>34.5</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="13.15" x14ac:dyDescent="0.4">

</xml_diff>

<commit_message>
Evita lo schermo nero quando una pagina non si carica
Se una pagina va in errore o il suo codice non si scarica (per esempio dopo un
aggiornamento del sito) l'app non si svuota più: compare un avviso con
"Ricarica la pagina", e per gli errori di caricamento del codice la pagina
si ricarica da sola, al massimo una volta ogni 10 secondi.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/libretti/manuel-bulla.xlsx
+++ b/docs/libretti/manuel-bulla.xlsx
@@ -770,8 +770,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F7E690B7-EC62-4BC2-A27A-E592475A3F24}" name="Registro" displayName="Registro" ref="A8:E31" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
-  <autoFilter ref="A8:E31" xr:uid="{F7E690B7-EC62-4BC2-A27A-E592475A3F24}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F7E690B7-EC62-4BC2-A27A-E592475A3F24}" name="Registro" displayName="Registro" ref="A8:E32" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
+  <autoFilter ref="A8:E32" xr:uid="{F7E690B7-EC62-4BC2-A27A-E592475A3F24}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
@@ -1575,21 +1575,44 @@
         <v>89</v>
       </c>
     </row>
+    <row r="32" spans="1:5" ht="25.5" x14ac:dyDescent="0.35">
+      <c r="A32" s="11">
+        <v>46310</v>
+      </c>
+      <c r="B32" s="10" t="inlineStr">
+        <is>
+          <t>Correzione dello schermo nero</t>
+        </is>
+      </c>
+      <c r="C32" s="12">
+        <v>1.5</v>
+      </c>
+      <c r="D32" s="9" t="inlineStr">
+        <is>
+          <t>Aggiunto un avviso con "Ricarica la pagina" quando una pagina va in errore e il ricaricamento automatico dopo un aggiornamento del sito, così non resta più lo schermo nero.</t>
+        </is>
+      </c>
+      <c r="E32" s="9" t="inlineStr">
+        <is>
+          <t>versione-corrente/frontend/src/components/ErroreImprevisto.jsx</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A7:E7"/>
   </mergeCells>
-  <conditionalFormatting sqref="C9:C31">
+  <conditionalFormatting sqref="C9:C32">
     <cfRule type="expression" dxfId="1" priority="1" stopIfTrue="1">
       <formula>($B9&lt;&gt;"")*($C9="")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Data non valida" error="Scrivi la data come gg/mm/aaaa, per esempio 14/10/2026." sqref="A9:A31" xr:uid="{D26B2BD8-0AFD-48FB-BBA1-B07F75408464}">
+    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Data non valida" error="Scrivi la data come gg/mm/aaaa, per esempio 14/10/2026." sqref="A9:A32" xr:uid="{D26B2BD8-0AFD-48FB-BBA1-B07F75408464}">
       <formula1>46023</formula1>
       <formula2>47483</formula2>
     </dataValidation>
-    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Ore non valide" error="Scrivi le ore come numero tra 0 e 24 (1,5 = un'ora e mezza)." promptTitle="Ore dedicate" prompt="Numero di ore, anche decimale: 1,5 = un'ora e mezza." sqref="C9:C31" xr:uid="{04EB0103-1D9C-4DFC-8906-92996DF6DE7A}">
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Ore non valide" error="Scrivi le ore come numero tra 0 e 24 (1,5 = un'ora e mezza)." promptTitle="Ore dedicate" prompt="Numero di ore, anche decimale: 1,5 = un'ora e mezza." sqref="C9:C32" xr:uid="{04EB0103-1D9C-4DFC-8906-92996DF6DE7A}">
       <formula1>0</formula1>
       <formula2>24</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
Libretto Manuel: pubblicazione su Google Cloud e HTTPS
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/libretti/manuel-bulla.xlsx
+++ b/docs/libretti/manuel-bulla.xlsx
@@ -770,8 +770,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F7E690B7-EC62-4BC2-A27A-E592475A3F24}" name="Registro" displayName="Registro" ref="A8:E32" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
-  <autoFilter ref="A8:E32" xr:uid="{F7E690B7-EC62-4BC2-A27A-E592475A3F24}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F7E690B7-EC62-4BC2-A27A-E592475A3F24}" name="Registro" displayName="Registro" ref="A8:E34" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
+  <autoFilter ref="A8:E34" xr:uid="{F7E690B7-EC62-4BC2-A27A-E592475A3F24}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
@@ -1598,21 +1598,67 @@
         </is>
       </c>
     </row>
+    <row r="33" spans="1:5" ht="25.5" x14ac:dyDescent="0.35">
+      <c r="A33" s="11">
+        <v>46310</v>
+      </c>
+      <c r="B33" s="10" t="inlineStr">
+        <is>
+          <t>Pubblicazione del sito su Google Cloud</t>
+        </is>
+      </c>
+      <c r="C33" s="12">
+        <v>3</v>
+      </c>
+      <c r="D33" s="9" t="inlineStr">
+        <is>
+          <t>Creata la macchina virtuale su Compute Engine (IP statico, firewall), installato Docker e avviato il sito con Docker Compose dal repository GitHub.</t>
+        </is>
+      </c>
+      <c r="E33" s="9" t="inlineStr">
+        <is>
+          <t>Progetto cgd-2026-disi-ingsoftware-mabu</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" spans="1:5" ht="25.5" x14ac:dyDescent="0.35">
+      <c r="A34" s="11">
+        <v>46310</v>
+      </c>
+      <c r="B34" s="10" t="inlineStr">
+        <is>
+          <t>Connessione sicura (HTTPS)</t>
+        </is>
+      </c>
+      <c r="C34" s="12">
+        <v>1</v>
+      </c>
+      <c r="D34" s="9" t="inlineStr">
+        <is>
+          <t>Attivato il proxy Caddy con certificato Let's Encrypt su 34-154-238-197.sslip.io: HTTP rimanda a HTTPS, con HSTS e porta 3000 chiusa.</t>
+        </is>
+      </c>
+      <c r="E34" s="9" t="inlineStr">
+        <is>
+          <t>https://34-154-238-197.sslip.io</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A7:E7"/>
   </mergeCells>
-  <conditionalFormatting sqref="C9:C32">
+  <conditionalFormatting sqref="C9:C34">
     <cfRule type="expression" dxfId="1" priority="1" stopIfTrue="1">
       <formula>($B9&lt;&gt;"")*($C9="")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Data non valida" error="Scrivi la data come gg/mm/aaaa, per esempio 14/10/2026." sqref="A9:A32" xr:uid="{D26B2BD8-0AFD-48FB-BBA1-B07F75408464}">
+    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Data non valida" error="Scrivi la data come gg/mm/aaaa, per esempio 14/10/2026." sqref="A9:A34" xr:uid="{D26B2BD8-0AFD-48FB-BBA1-B07F75408464}">
       <formula1>46023</formula1>
       <formula2>47483</formula2>
     </dataValidation>
-    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Ore non valide" error="Scrivi le ore come numero tra 0 e 24 (1,5 = un'ora e mezza)." promptTitle="Ore dedicate" prompt="Numero di ore, anche decimale: 1,5 = un'ora e mezza." sqref="C9:C32" xr:uid="{04EB0103-1D9C-4DFC-8906-92996DF6DE7A}">
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Ore non valide" error="Scrivi le ore come numero tra 0 e 24 (1,5 = un'ora e mezza)." promptTitle="Ore dedicate" prompt="Numero di ore, anche decimale: 1,5 = un'ora e mezza." sqref="C9:C34" xr:uid="{04EB0103-1D9C-4DFC-8906-92996DF6DE7A}">
       <formula1>0</formula1>
       <formula2>24</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
Archivia il frontend v3 tra le versioni precedenti
Copia autonoma del frontend corrente in versioni-precedenti/frontend-v3 (porta 5177, test propri,
npm run dev:v3), con contenuti in tre lingue, mappa MapTiler e vista satellitare.
README e libretto di Manuel aggiornati.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/libretti/manuel-bulla.xlsx
+++ b/docs/libretti/manuel-bulla.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bulla\Documents\Ing-software-v1\docs\libretti\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C69A8E71-3EB6-4B3F-B117-231ACE64114D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBE73731-F703-4E91-B3EB-906E5C761571}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{EB300ADB-58B5-479D-B51B-E912DFEACD78}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="102">
   <si>
     <t>Libretto delle attività</t>
   </si>
@@ -313,6 +313,42 @@
   </si>
   <si>
     <t>versione-corrente/frontend/src/components/MappaLeaflet.jsx, lib/sfondo.js, stile.css, i18n</t>
+  </si>
+  <si>
+    <t>Correzione dello schermo nero</t>
+  </si>
+  <si>
+    <t>Aggiunto un avviso con "Ricarica la pagina" quando una pagina va in errore e il ricaricamento automatico dopo un aggiornamento del sito, così non resta più lo schermo nero.</t>
+  </si>
+  <si>
+    <t>versione-corrente/frontend/src/components/ErroreImprevisto.jsx</t>
+  </si>
+  <si>
+    <t>Pubblicazione del sito su Google Cloud</t>
+  </si>
+  <si>
+    <t>Creata la macchina virtuale su Compute Engine (IP statico, firewall), installato Docker e avviato il sito con Docker Compose dal repository GitHub.</t>
+  </si>
+  <si>
+    <t>Progetto cgd-2026-disi-ingsoftware-mabu</t>
+  </si>
+  <si>
+    <t>Connessione sicura (HTTPS)</t>
+  </si>
+  <si>
+    <t>Attivato il proxy Caddy con certificato Let's Encrypt su 34-154-238-197.sslip.io: HTTP rimanda a HTTPS, con HSTS e porta 3000 chiusa.</t>
+  </si>
+  <si>
+    <t>https://34-154-238-197.sslip.io</t>
+  </si>
+  <si>
+    <t>Archivio del frontend v3</t>
+  </si>
+  <si>
+    <t>Copia autonoma del frontend corrente in versioni-precedenti (porta 5177, test propri, npm run dev:v3), con README e documenti aggiornati.</t>
+  </si>
+  <si>
+    <t>versioni-precedenti/frontend-v3/, README.md, CONTRIBUTING.md, package.json</t>
   </si>
 </sst>
 </file>
@@ -770,8 +806,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F7E690B7-EC62-4BC2-A27A-E592475A3F24}" name="Registro" displayName="Registro" ref="A8:E34" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
-  <autoFilter ref="A8:E34" xr:uid="{F7E690B7-EC62-4BC2-A27A-E592475A3F24}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F7E690B7-EC62-4BC2-A27A-E592475A3F24}" name="Registro" displayName="Registro" ref="A8:E35" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
+  <autoFilter ref="A8:E35" xr:uid="{F7E690B7-EC62-4BC2-A27A-E592475A3F24}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
@@ -1109,7 +1145,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.59765625" style="1" customWidth="1"/>
@@ -1146,7 +1182,7 @@
       </c>
       <c r="C5" s="7">
         <f>SUM(Registro[Ore])</f>
-        <v>34.5</v>
+        <v>41</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="13.15" x14ac:dyDescent="0.4">
@@ -1575,90 +1611,89 @@
         <v>89</v>
       </c>
     </row>
-    <row r="32" spans="1:5" ht="25.5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:5" ht="38.25" x14ac:dyDescent="0.35">
       <c r="A32" s="11">
         <v>46310</v>
       </c>
-      <c r="B32" s="10" t="inlineStr">
-        <is>
-          <t>Correzione dello schermo nero</t>
-        </is>
+      <c r="B32" s="10" t="s">
+        <v>90</v>
       </c>
       <c r="C32" s="12">
         <v>1.5</v>
       </c>
-      <c r="D32" s="9" t="inlineStr">
-        <is>
-          <t>Aggiunto un avviso con "Ricarica la pagina" quando una pagina va in errore e il ricaricamento automatico dopo un aggiornamento del sito, così non resta più lo schermo nero.</t>
-        </is>
-      </c>
-      <c r="E32" s="9" t="inlineStr">
-        <is>
-          <t>versione-corrente/frontend/src/components/ErroreImprevisto.jsx</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" spans="1:5" ht="25.5" x14ac:dyDescent="0.35">
+      <c r="D32" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="E32" s="9" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" ht="26.25" x14ac:dyDescent="0.35">
       <c r="A33" s="11">
         <v>46310</v>
       </c>
-      <c r="B33" s="10" t="inlineStr">
-        <is>
-          <t>Pubblicazione del sito su Google Cloud</t>
-        </is>
+      <c r="B33" s="10" t="s">
+        <v>93</v>
       </c>
       <c r="C33" s="12">
         <v>3</v>
       </c>
-      <c r="D33" s="9" t="inlineStr">
-        <is>
-          <t>Creata la macchina virtuale su Compute Engine (IP statico, firewall), installato Docker e avviato il sito con Docker Compose dal repository GitHub.</t>
-        </is>
-      </c>
-      <c r="E33" s="9" t="inlineStr">
-        <is>
-          <t>Progetto cgd-2026-disi-ingsoftware-mabu</t>
-        </is>
+      <c r="D33" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="E33" s="9" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="34" spans="1:5" ht="25.5" x14ac:dyDescent="0.35">
       <c r="A34" s="11">
         <v>46310</v>
       </c>
-      <c r="B34" s="10" t="inlineStr">
-        <is>
-          <t>Connessione sicura (HTTPS)</t>
-        </is>
+      <c r="B34" s="10" t="s">
+        <v>96</v>
       </c>
       <c r="C34" s="12">
         <v>1</v>
       </c>
-      <c r="D34" s="9" t="inlineStr">
-        <is>
-          <t>Attivato il proxy Caddy con certificato Let's Encrypt su 34-154-238-197.sslip.io: HTTP rimanda a HTTPS, con HSTS e porta 3000 chiusa.</t>
-        </is>
-      </c>
-      <c r="E34" s="9" t="inlineStr">
-        <is>
-          <t>https://34-154-238-197.sslip.io</t>
-        </is>
+      <c r="D34" s="9" t="s">
+        <v>97</v>
+      </c>
+      <c r="E34" s="9" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" ht="25.5" x14ac:dyDescent="0.35">
+      <c r="A35" s="11">
+        <v>46310</v>
+      </c>
+      <c r="B35" s="10" t="s">
+        <v>99</v>
+      </c>
+      <c r="C35" s="12">
+        <v>1</v>
+      </c>
+      <c r="D35" s="9" t="s">
+        <v>100</v>
+      </c>
+      <c r="E35" s="9" t="s">
+        <v>101</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A7:E7"/>
   </mergeCells>
-  <conditionalFormatting sqref="C9:C34">
+  <conditionalFormatting sqref="C9:C35">
     <cfRule type="expression" dxfId="1" priority="1" stopIfTrue="1">
       <formula>($B9&lt;&gt;"")*($C9="")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Data non valida" error="Scrivi la data come gg/mm/aaaa, per esempio 14/10/2026." sqref="A9:A34" xr:uid="{D26B2BD8-0AFD-48FB-BBA1-B07F75408464}">
+    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Data non valida" error="Scrivi la data come gg/mm/aaaa, per esempio 14/10/2026." sqref="A9:A35" xr:uid="{D26B2BD8-0AFD-48FB-BBA1-B07F75408464}">
       <formula1>46023</formula1>
       <formula2>47483</formula2>
     </dataValidation>
-    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Ore non valide" error="Scrivi le ore come numero tra 0 e 24 (1,5 = un'ora e mezza)." promptTitle="Ore dedicate" prompt="Numero di ore, anche decimale: 1,5 = un'ora e mezza." sqref="C9:C34" xr:uid="{04EB0103-1D9C-4DFC-8906-92996DF6DE7A}">
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Ore non valide" error="Scrivi le ore come numero tra 0 e 24 (1,5 = un'ora e mezza)." promptTitle="Ore dedicate" prompt="Numero di ore, anche decimale: 1,5 = un'ora e mezza." sqref="C9:C35" xr:uid="{04EB0103-1D9C-4DFC-8906-92996DF6DE7A}">
       <formula1>0</formula1>
       <formula2>24</formula2>
     </dataValidation>
@@ -1780,15 +1815,15 @@
       </c>
       <c r="C8" s="19">
         <f>COUNTIFS(Registro[Data],"&gt;="&amp;A8,Registro[Data],"&lt;="&amp;B8)</f>
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="D8" s="20">
         <f>SUMIFS(Registro[Ore],Registro[Data],"&gt;="&amp;A8,Registro[Data],"&lt;="&amp;B8)</f>
-        <v>8.5</v>
+        <v>15</v>
       </c>
       <c r="E8" s="20">
         <f>SUM(D$6:D8)</f>
-        <v>34.5</v>
+        <v>41</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
@@ -1810,7 +1845,7 @@
       </c>
       <c r="E9" s="23">
         <f>SUM(D$6:D9)</f>
-        <v>34.5</v>
+        <v>41</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
@@ -1832,7 +1867,7 @@
       </c>
       <c r="E10" s="20">
         <f>SUM(D$6:D10)</f>
-        <v>34.5</v>
+        <v>41</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.35">
@@ -1854,7 +1889,7 @@
       </c>
       <c r="E11" s="23">
         <f>SUM(D$6:D11)</f>
-        <v>34.5</v>
+        <v>41</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.35">
@@ -1876,7 +1911,7 @@
       </c>
       <c r="E12" s="20">
         <f>SUM(D$6:D12)</f>
-        <v>34.5</v>
+        <v>41</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
@@ -1898,7 +1933,7 @@
       </c>
       <c r="E13" s="23">
         <f>SUM(D$6:D13)</f>
-        <v>34.5</v>
+        <v>41</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
@@ -1920,7 +1955,7 @@
       </c>
       <c r="E14" s="20">
         <f>SUM(D$6:D14)</f>
-        <v>34.5</v>
+        <v>41</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.35">
@@ -1942,7 +1977,7 @@
       </c>
       <c r="E15" s="23">
         <f>SUM(D$6:D15)</f>
-        <v>34.5</v>
+        <v>41</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.35">
@@ -1964,7 +1999,7 @@
       </c>
       <c r="E16" s="20">
         <f>SUM(D$6:D16)</f>
-        <v>34.5</v>
+        <v>41</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.35">
@@ -1986,7 +2021,7 @@
       </c>
       <c r="E17" s="23">
         <f>SUM(D$6:D17)</f>
-        <v>34.5</v>
+        <v>41</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.35">
@@ -2008,7 +2043,7 @@
       </c>
       <c r="E18" s="20">
         <f>SUM(D$6:D18)</f>
-        <v>34.5</v>
+        <v>41</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.35">
@@ -2030,7 +2065,7 @@
       </c>
       <c r="E19" s="23">
         <f>SUM(D$6:D19)</f>
-        <v>34.5</v>
+        <v>41</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.35">
@@ -2052,7 +2087,7 @@
       </c>
       <c r="E20" s="20">
         <f>SUM(D$6:D20)</f>
-        <v>34.5</v>
+        <v>41</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.35">
@@ -2074,7 +2109,7 @@
       </c>
       <c r="E21" s="26">
         <f>SUM(D$6:D21)</f>
-        <v>34.5</v>
+        <v>41</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="13.15" x14ac:dyDescent="0.4">
@@ -2084,11 +2119,11 @@
       <c r="B22" s="28"/>
       <c r="C22" s="29">
         <f>SUM(C6:C21)</f>
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="D22" s="30">
         <f>SUM(D6:D21)</f>
-        <v>34.5</v>
+        <v>41</v>
       </c>
       <c r="E22" s="28"/>
     </row>
@@ -2100,7 +2135,7 @@
       <c r="C24" s="6"/>
       <c r="D24" s="15">
         <f>SUM(Registro[Ore])</f>
-        <v>34.5</v>
+        <v>41</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="13.15" x14ac:dyDescent="0.4">

</xml_diff>

<commit_message>
Libretto Manuel: ore ridotte per le voci piccole
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/libretti/manuel-bulla.xlsx
+++ b/docs/libretti/manuel-bulla.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bulla\Documents\Ing-software-v1\docs\libretti\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBE73731-F703-4E91-B3EB-906E5C761571}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB3C1335-6172-4FE9-B31A-B34475DCCB0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{EB300ADB-58B5-479D-B51B-E912DFEACD78}"/>
   </bookViews>
@@ -1182,7 +1182,7 @@
       </c>
       <c r="C5" s="7">
         <f>SUM(Registro[Ore])</f>
-        <v>41</v>
+        <v>39.5</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="13.15" x14ac:dyDescent="0.4">
@@ -1585,7 +1585,7 @@
         <v>84</v>
       </c>
       <c r="C30" s="12">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="D30" s="9" t="s">
         <v>85</v>
@@ -1602,7 +1602,7 @@
         <v>87</v>
       </c>
       <c r="C31" s="12">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="D31" s="9" t="s">
         <v>88</v>
@@ -1670,7 +1670,7 @@
         <v>99</v>
       </c>
       <c r="C35" s="12">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="D35" s="9" t="s">
         <v>100</v>
@@ -1819,11 +1819,11 @@
       </c>
       <c r="D8" s="20">
         <f>SUMIFS(Registro[Ore],Registro[Data],"&gt;="&amp;A8,Registro[Data],"&lt;="&amp;B8)</f>
-        <v>15</v>
+        <v>13.5</v>
       </c>
       <c r="E8" s="20">
         <f>SUM(D$6:D8)</f>
-        <v>41</v>
+        <v>39.5</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
@@ -1845,7 +1845,7 @@
       </c>
       <c r="E9" s="23">
         <f>SUM(D$6:D9)</f>
-        <v>41</v>
+        <v>39.5</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
@@ -1867,7 +1867,7 @@
       </c>
       <c r="E10" s="20">
         <f>SUM(D$6:D10)</f>
-        <v>41</v>
+        <v>39.5</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.35">
@@ -1889,7 +1889,7 @@
       </c>
       <c r="E11" s="23">
         <f>SUM(D$6:D11)</f>
-        <v>41</v>
+        <v>39.5</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.35">
@@ -1911,7 +1911,7 @@
       </c>
       <c r="E12" s="20">
         <f>SUM(D$6:D12)</f>
-        <v>41</v>
+        <v>39.5</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
@@ -1933,7 +1933,7 @@
       </c>
       <c r="E13" s="23">
         <f>SUM(D$6:D13)</f>
-        <v>41</v>
+        <v>39.5</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
@@ -1955,7 +1955,7 @@
       </c>
       <c r="E14" s="20">
         <f>SUM(D$6:D14)</f>
-        <v>41</v>
+        <v>39.5</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.35">
@@ -1977,7 +1977,7 @@
       </c>
       <c r="E15" s="23">
         <f>SUM(D$6:D15)</f>
-        <v>41</v>
+        <v>39.5</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.35">
@@ -1999,7 +1999,7 @@
       </c>
       <c r="E16" s="20">
         <f>SUM(D$6:D16)</f>
-        <v>41</v>
+        <v>39.5</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.35">
@@ -2021,7 +2021,7 @@
       </c>
       <c r="E17" s="23">
         <f>SUM(D$6:D17)</f>
-        <v>41</v>
+        <v>39.5</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.35">
@@ -2043,7 +2043,7 @@
       </c>
       <c r="E18" s="20">
         <f>SUM(D$6:D18)</f>
-        <v>41</v>
+        <v>39.5</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.35">
@@ -2065,7 +2065,7 @@
       </c>
       <c r="E19" s="23">
         <f>SUM(D$6:D19)</f>
-        <v>41</v>
+        <v>39.5</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.35">
@@ -2087,7 +2087,7 @@
       </c>
       <c r="E20" s="20">
         <f>SUM(D$6:D20)</f>
-        <v>41</v>
+        <v>39.5</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.35">
@@ -2109,7 +2109,7 @@
       </c>
       <c r="E21" s="26">
         <f>SUM(D$6:D21)</f>
-        <v>41</v>
+        <v>39.5</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="13.15" x14ac:dyDescent="0.4">
@@ -2123,7 +2123,7 @@
       </c>
       <c r="D22" s="30">
         <f>SUM(D6:D21)</f>
-        <v>41</v>
+        <v>39.5</v>
       </c>
       <c r="E22" s="28"/>
     </row>
@@ -2135,7 +2135,7 @@
       <c r="C24" s="6"/>
       <c r="D24" s="15">
         <f>SUM(Registro[Ore])</f>
-        <v>41</v>
+        <v>39.5</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="13.15" x14ac:dyDescent="0.4">

</xml_diff>

<commit_message>
Libretto Manuel: dominio gratuito e posta con Brevo
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/libretti/manuel-bulla.xlsx
+++ b/docs/libretti/manuel-bulla.xlsx
@@ -806,8 +806,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F7E690B7-EC62-4BC2-A27A-E592475A3F24}" name="Registro" displayName="Registro" ref="A8:E35" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
-  <autoFilter ref="A8:E35" xr:uid="{F7E690B7-EC62-4BC2-A27A-E592475A3F24}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F7E690B7-EC62-4BC2-A27A-E592475A3F24}" name="Registro" displayName="Registro" ref="A8:E36" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
+  <autoFilter ref="A8:E36" xr:uid="{F7E690B7-EC62-4BC2-A27A-E592475A3F24}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
@@ -1679,21 +1679,44 @@
         <v>101</v>
       </c>
     </row>
+    <row r="36" spans="1:5" ht="25.5" x14ac:dyDescent="0.35">
+      <c r="A36" s="11">
+        <v>46310</v>
+      </c>
+      <c r="B36" s="10" t="inlineStr">
+        <is>
+          <t>Dominio e posta del sito</t>
+        </is>
+      </c>
+      <c r="C36" s="12">
+        <v>1.5</v>
+      </c>
+      <c r="D36" s="9" t="inlineStr">
+        <is>
+          <t>Dominio gratuito discover-tridentum.duckdns.org con HTTPS e invio delle e-mail di conferma tramite Brevo (SMTP), provato con una mail di prova.</t>
+        </is>
+      </c>
+      <c r="E36" s="9" t="inlineStr">
+        <is>
+          <t>https://discover-tridentum.duckdns.org</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A7:E7"/>
   </mergeCells>
-  <conditionalFormatting sqref="C9:C35">
+  <conditionalFormatting sqref="C9:C36">
     <cfRule type="expression" dxfId="1" priority="1" stopIfTrue="1">
       <formula>($B9&lt;&gt;"")*($C9="")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Data non valida" error="Scrivi la data come gg/mm/aaaa, per esempio 14/10/2026." sqref="A9:A35" xr:uid="{D26B2BD8-0AFD-48FB-BBA1-B07F75408464}">
+    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Data non valida" error="Scrivi la data come gg/mm/aaaa, per esempio 14/10/2026." sqref="A9:A36" xr:uid="{D26B2BD8-0AFD-48FB-BBA1-B07F75408464}">
       <formula1>46023</formula1>
       <formula2>47483</formula2>
     </dataValidation>
-    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Ore non valide" error="Scrivi le ore come numero tra 0 e 24 (1,5 = un'ora e mezza)." promptTitle="Ore dedicate" prompt="Numero di ore, anche decimale: 1,5 = un'ora e mezza." sqref="C9:C35" xr:uid="{04EB0103-1D9C-4DFC-8906-92996DF6DE7A}">
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Ore non valide" error="Scrivi le ore come numero tra 0 e 24 (1,5 = un'ora e mezza)." promptTitle="Ore dedicate" prompt="Numero di ore, anche decimale: 1,5 = un'ora e mezza." sqref="C9:C36" xr:uid="{04EB0103-1D9C-4DFC-8906-92996DF6DE7A}">
       <formula1>0</formula1>
       <formula2>24</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
Aggiorna l'elenco dei compiti dopo un nuovo controllo del sito
Controllati versione corrente e sito pubblicato dopo le ultime modifiche
(tedesco, mappa MapTiler e satellite, galleria del benvenuto, Google Cloud).

- Tolti i compiti fatti: HTTPS sul sito pubblicato, avvio con un solo comando,
  indirizzo per la privacy impostato sul server e dati del titolare nell'informativa
- Aggiornate le situazioni degli altri compiti (foto, browser, accessibilita',
  carico, Fase 2, Fase 3, verifica, fornitori, copie di sicurezza)
- Aggiunti tre compiti: galleria del benvenuto, sito pubblicato e chiave MapTiler
- Corrette le formule "Per persona" del Riepilogo, che contavano la colonna
  "Situazione attuale" invece di "Assegnato a"
- Voce nel libretto di Manuel

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/libretti/manuel-bulla.xlsx
+++ b/docs/libretti/manuel-bulla.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bulla\Documents\Ing-software-v1\docs\libretti\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB3C1335-6172-4FE9-B31A-B34475DCCB0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB39AB5D-58FB-43A0-A16F-89E7ABB21BD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{EB300ADB-58B5-479D-B51B-E912DFEACD78}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="107">
   <si>
     <t>Libretto delle attività</t>
   </si>
@@ -349,6 +349,21 @@
   </si>
   <si>
     <t>versioni-precedenti/frontend-v3/, README.md, CONTRIBUTING.md, package.json</t>
+  </si>
+  <si>
+    <t>Dominio e posta del sito</t>
+  </si>
+  <si>
+    <t>Dominio gratuito discover-tridentum.duckdns.org con HTTPS e invio delle e-mail di conferma tramite Brevo (SMTP), provato con una mail di prova.</t>
+  </si>
+  <si>
+    <t>https://discover-tridentum.duckdns.org</t>
+  </si>
+  <si>
+    <t>Terzo controllo del sito e aggiornamento dei compiti</t>
+  </si>
+  <si>
+    <t>Nuovo controllo dopo le ultime modifiche (tedesco, satellite, galleria, sito online): 4 compiti chiusi, 3 nuovi, gli altri aggiornati; corretto il Riepilogo.</t>
   </si>
 </sst>
 </file>
@@ -806,8 +821,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F7E690B7-EC62-4BC2-A27A-E592475A3F24}" name="Registro" displayName="Registro" ref="A8:E36" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
-  <autoFilter ref="A8:E36" xr:uid="{F7E690B7-EC62-4BC2-A27A-E592475A3F24}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F7E690B7-EC62-4BC2-A27A-E592475A3F24}" name="Registro" displayName="Registro" ref="A8:E37" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
+  <autoFilter ref="A8:E37" xr:uid="{F7E690B7-EC62-4BC2-A27A-E592475A3F24}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
@@ -1145,7 +1160,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.59765625" style="1" customWidth="1"/>
@@ -1182,7 +1197,7 @@
       </c>
       <c r="C5" s="7">
         <f>SUM(Registro[Ore])</f>
-        <v>39.5</v>
+        <v>43.5</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="13.15" x14ac:dyDescent="0.4">
@@ -1683,40 +1698,51 @@
       <c r="A36" s="11">
         <v>46310</v>
       </c>
-      <c r="B36" s="10" t="inlineStr">
-        <is>
-          <t>Dominio e posta del sito</t>
-        </is>
+      <c r="B36" s="10" t="s">
+        <v>102</v>
       </c>
       <c r="C36" s="12">
         <v>1.5</v>
       </c>
-      <c r="D36" s="9" t="inlineStr">
-        <is>
-          <t>Dominio gratuito discover-tridentum.duckdns.org con HTTPS e invio delle e-mail di conferma tramite Brevo (SMTP), provato con una mail di prova.</t>
-        </is>
-      </c>
-      <c r="E36" s="9" t="inlineStr">
-        <is>
-          <t>https://discover-tridentum.duckdns.org</t>
-        </is>
+      <c r="D36" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="E36" s="9" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" ht="26.25" x14ac:dyDescent="0.35">
+      <c r="A37" s="11">
+        <v>46311</v>
+      </c>
+      <c r="B37" s="10" t="s">
+        <v>105</v>
+      </c>
+      <c r="C37" s="12">
+        <v>2.5</v>
+      </c>
+      <c r="D37" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="E37" s="9" t="s">
+        <v>80</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A7:E7"/>
   </mergeCells>
-  <conditionalFormatting sqref="C9:C36">
+  <conditionalFormatting sqref="C9:C37">
     <cfRule type="expression" dxfId="1" priority="1" stopIfTrue="1">
       <formula>($B9&lt;&gt;"")*($C9="")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Data non valida" error="Scrivi la data come gg/mm/aaaa, per esempio 14/10/2026." sqref="A9:A36" xr:uid="{D26B2BD8-0AFD-48FB-BBA1-B07F75408464}">
+    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Data non valida" error="Scrivi la data come gg/mm/aaaa, per esempio 14/10/2026." sqref="A9:A37" xr:uid="{D26B2BD8-0AFD-48FB-BBA1-B07F75408464}">
       <formula1>46023</formula1>
       <formula2>47483</formula2>
     </dataValidation>
-    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Ore non valide" error="Scrivi le ore come numero tra 0 e 24 (1,5 = un'ora e mezza)." promptTitle="Ore dedicate" prompt="Numero di ore, anche decimale: 1,5 = un'ora e mezza." sqref="C9:C36" xr:uid="{04EB0103-1D9C-4DFC-8906-92996DF6DE7A}">
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Ore non valide" error="Scrivi le ore come numero tra 0 e 24 (1,5 = un'ora e mezza)." promptTitle="Ore dedicate" prompt="Numero di ore, anche decimale: 1,5 = un'ora e mezza." sqref="C9:C37" xr:uid="{04EB0103-1D9C-4DFC-8906-92996DF6DE7A}">
       <formula1>0</formula1>
       <formula2>24</formula2>
     </dataValidation>
@@ -1838,15 +1864,15 @@
       </c>
       <c r="C8" s="19">
         <f>COUNTIFS(Registro[Data],"&gt;="&amp;A8,Registro[Data],"&lt;="&amp;B8)</f>
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D8" s="20">
         <f>SUMIFS(Registro[Ore],Registro[Data],"&gt;="&amp;A8,Registro[Data],"&lt;="&amp;B8)</f>
-        <v>13.5</v>
+        <v>17.5</v>
       </c>
       <c r="E8" s="20">
         <f>SUM(D$6:D8)</f>
-        <v>39.5</v>
+        <v>43.5</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
@@ -1868,7 +1894,7 @@
       </c>
       <c r="E9" s="23">
         <f>SUM(D$6:D9)</f>
-        <v>39.5</v>
+        <v>43.5</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
@@ -1890,7 +1916,7 @@
       </c>
       <c r="E10" s="20">
         <f>SUM(D$6:D10)</f>
-        <v>39.5</v>
+        <v>43.5</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.35">
@@ -1912,7 +1938,7 @@
       </c>
       <c r="E11" s="23">
         <f>SUM(D$6:D11)</f>
-        <v>39.5</v>
+        <v>43.5</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.35">
@@ -1934,7 +1960,7 @@
       </c>
       <c r="E12" s="20">
         <f>SUM(D$6:D12)</f>
-        <v>39.5</v>
+        <v>43.5</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
@@ -1956,7 +1982,7 @@
       </c>
       <c r="E13" s="23">
         <f>SUM(D$6:D13)</f>
-        <v>39.5</v>
+        <v>43.5</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
@@ -1978,7 +2004,7 @@
       </c>
       <c r="E14" s="20">
         <f>SUM(D$6:D14)</f>
-        <v>39.5</v>
+        <v>43.5</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.35">
@@ -2000,7 +2026,7 @@
       </c>
       <c r="E15" s="23">
         <f>SUM(D$6:D15)</f>
-        <v>39.5</v>
+        <v>43.5</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.35">
@@ -2022,7 +2048,7 @@
       </c>
       <c r="E16" s="20">
         <f>SUM(D$6:D16)</f>
-        <v>39.5</v>
+        <v>43.5</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.35">
@@ -2044,7 +2070,7 @@
       </c>
       <c r="E17" s="23">
         <f>SUM(D$6:D17)</f>
-        <v>39.5</v>
+        <v>43.5</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.35">
@@ -2066,7 +2092,7 @@
       </c>
       <c r="E18" s="20">
         <f>SUM(D$6:D18)</f>
-        <v>39.5</v>
+        <v>43.5</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.35">
@@ -2088,7 +2114,7 @@
       </c>
       <c r="E19" s="23">
         <f>SUM(D$6:D19)</f>
-        <v>39.5</v>
+        <v>43.5</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.35">
@@ -2110,7 +2136,7 @@
       </c>
       <c r="E20" s="20">
         <f>SUM(D$6:D20)</f>
-        <v>39.5</v>
+        <v>43.5</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.35">
@@ -2132,7 +2158,7 @@
       </c>
       <c r="E21" s="26">
         <f>SUM(D$6:D21)</f>
-        <v>39.5</v>
+        <v>43.5</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="13.15" x14ac:dyDescent="0.4">
@@ -2142,11 +2168,11 @@
       <c r="B22" s="28"/>
       <c r="C22" s="29">
         <f>SUM(C6:C21)</f>
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D22" s="30">
         <f>SUM(D6:D21)</f>
-        <v>39.5</v>
+        <v>43.5</v>
       </c>
       <c r="E22" s="28"/>
     </row>
@@ -2158,7 +2184,7 @@
       <c r="C24" s="6"/>
       <c r="D24" s="15">
         <f>SUM(Registro[Ore])</f>
-        <v>39.5</v>
+        <v>43.5</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="13.15" x14ac:dyDescent="0.4">

</xml_diff>

<commit_message>
Libretti: riunione del team (1 ora ciascuno)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/libretti/manuel-bulla.xlsx
+++ b/docs/libretti/manuel-bulla.xlsx
@@ -821,8 +821,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F7E690B7-EC62-4BC2-A27A-E592475A3F24}" name="Registro" displayName="Registro" ref="A8:E37" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
-  <autoFilter ref="A8:E37" xr:uid="{F7E690B7-EC62-4BC2-A27A-E592475A3F24}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F7E690B7-EC62-4BC2-A27A-E592475A3F24}" name="Registro" displayName="Registro" ref="A8:E38" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
+  <autoFilter ref="A8:E38" xr:uid="{F7E690B7-EC62-4BC2-A27A-E592475A3F24}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
@@ -1728,21 +1728,44 @@
         <v>80</v>
       </c>
     </row>
+    <row r="38" spans="1:5" ht="25.5" x14ac:dyDescent="0.35">
+      <c r="A38" s="11">
+        <v>46311</v>
+      </c>
+      <c r="B38" s="10" t="inlineStr">
+        <is>
+          <t>Riunione del team</t>
+        </is>
+      </c>
+      <c r="C38" s="12">
+        <v>1</v>
+      </c>
+      <c r="D38" s="9" t="inlineStr">
+        <is>
+          <t>Riunione con tutto il team per fare il punto sul progetto e decidere i prossimi compiti.</t>
+        </is>
+      </c>
+      <c r="E38" s="9" t="inlineStr">
+        <is>
+          <t>Riunione del team</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A7:E7"/>
   </mergeCells>
-  <conditionalFormatting sqref="C9:C37">
+  <conditionalFormatting sqref="C9:C38">
     <cfRule type="expression" dxfId="1" priority="1" stopIfTrue="1">
       <formula>($B9&lt;&gt;"")*($C9="")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Data non valida" error="Scrivi la data come gg/mm/aaaa, per esempio 14/10/2026." sqref="A9:A37" xr:uid="{D26B2BD8-0AFD-48FB-BBA1-B07F75408464}">
+    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Data non valida" error="Scrivi la data come gg/mm/aaaa, per esempio 14/10/2026." sqref="A9:A38" xr:uid="{D26B2BD8-0AFD-48FB-BBA1-B07F75408464}">
       <formula1>46023</formula1>
       <formula2>47483</formula2>
     </dataValidation>
-    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Ore non valide" error="Scrivi le ore come numero tra 0 e 24 (1,5 = un'ora e mezza)." promptTitle="Ore dedicate" prompt="Numero di ore, anche decimale: 1,5 = un'ora e mezza." sqref="C9:C37" xr:uid="{04EB0103-1D9C-4DFC-8906-92996DF6DE7A}">
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Ore non valide" error="Scrivi le ore come numero tra 0 e 24 (1,5 = un'ora e mezza)." promptTitle="Ore dedicate" prompt="Numero di ore, anche decimale: 1,5 = un'ora e mezza." sqref="C9:C38" xr:uid="{04EB0103-1D9C-4DFC-8906-92996DF6DE7A}">
       <formula1>0</formula1>
       <formula2>24</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
Mappa con Google Maps (Map Tiles API)
Lo sfondo della mappa e la vista satellitare usano le tessere di Google Maps: il
browser chiede una sessione a Google e la tiene fino alla scadenza. La chiave sta
in VITE_GOOGLE_MAPS_KEY (build Docker, frontend/.env.local in sviluppo) ed è
limitata al dominio del sito e alla sola Map Tiles API. Senza chiave, o se Google
non risponde, si ripiega su OpenStreetMap ed Esri; le anteprime dei luoghi restano
su OpenStreetMap per non consumare la quota. Tolto MapTiler. Aggiornati
informativa privacy, regole CSP, decisione D-07 e documentazione.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/libretti/manuel-bulla.xlsx
+++ b/docs/libretti/manuel-bulla.xlsx
@@ -821,8 +821,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F7E690B7-EC62-4BC2-A27A-E592475A3F24}" name="Registro" displayName="Registro" ref="A8:E38" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
-  <autoFilter ref="A8:E38" xr:uid="{F7E690B7-EC62-4BC2-A27A-E592475A3F24}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F7E690B7-EC62-4BC2-A27A-E592475A3F24}" name="Registro" displayName="Registro" ref="A8:E39" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
+  <autoFilter ref="A8:E39" xr:uid="{F7E690B7-EC62-4BC2-A27A-E592475A3F24}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
@@ -1751,21 +1751,44 @@
         </is>
       </c>
     </row>
+    <row r="39" spans="1:5" ht="25.5" x14ac:dyDescent="0.35">
+      <c r="A39" s="11">
+        <v>46311</v>
+      </c>
+      <c r="B39" s="10" t="inlineStr">
+        <is>
+          <t>Mappa con Google Maps</t>
+        </is>
+      </c>
+      <c r="C39" s="12">
+        <v>3</v>
+      </c>
+      <c r="D39" s="9" t="inlineStr">
+        <is>
+          <t>Sfondo della mappa e vista satellitare con le tessere di Google Maps (Map Tiles API): chiave su Google Cloud limitata al dominio, ripiego su OpenStreetMap, informativa privacy e regole di sicurezza aggiornate.</t>
+        </is>
+      </c>
+      <c r="E39" s="9" t="inlineStr">
+        <is>
+          <t>versione-corrente/frontend/src/lib/sfondo.js</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A7:E7"/>
   </mergeCells>
-  <conditionalFormatting sqref="C9:C38">
+  <conditionalFormatting sqref="C9:C39">
     <cfRule type="expression" dxfId="1" priority="1" stopIfTrue="1">
       <formula>($B9&lt;&gt;"")*($C9="")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Data non valida" error="Scrivi la data come gg/mm/aaaa, per esempio 14/10/2026." sqref="A9:A38" xr:uid="{D26B2BD8-0AFD-48FB-BBA1-B07F75408464}">
+    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Data non valida" error="Scrivi la data come gg/mm/aaaa, per esempio 14/10/2026." sqref="A9:A39" xr:uid="{D26B2BD8-0AFD-48FB-BBA1-B07F75408464}">
       <formula1>46023</formula1>
       <formula2>47483</formula2>
     </dataValidation>
-    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Ore non valide" error="Scrivi le ore come numero tra 0 e 24 (1,5 = un'ora e mezza)." promptTitle="Ore dedicate" prompt="Numero di ore, anche decimale: 1,5 = un'ora e mezza." sqref="C9:C38" xr:uid="{04EB0103-1D9C-4DFC-8906-92996DF6DE7A}">
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Ore non valide" error="Scrivi le ore come numero tra 0 e 24 (1,5 = un'ora e mezza)." promptTitle="Ore dedicate" prompt="Numero di ore, anche decimale: 1,5 = un'ora e mezza." sqref="C9:C39" xr:uid="{04EB0103-1D9C-4DFC-8906-92996DF6DE7A}">
       <formula1>0</formula1>
       <formula2>24</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
Tolto il documento di verifica dei requisiti e ogni riferimento a MapTiler
Il documento sulla verifica dei requisiti non funzionali è sostituito dall'elenco dei
compiti (docs/compiti.xlsx). La mappa usa solo Google Maps: aggiornati README,
decisione D-07 e gli script di prestazioni.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/libretti/manuel-bulla.xlsx
+++ b/docs/libretti/manuel-bulla.xlsx
@@ -821,8 +821,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F7E690B7-EC62-4BC2-A27A-E592475A3F24}" name="Registro" displayName="Registro" ref="A8:E39" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
-  <autoFilter ref="A8:E39" xr:uid="{F7E690B7-EC62-4BC2-A27A-E592475A3F24}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F7E690B7-EC62-4BC2-A27A-E592475A3F24}" name="Registro" displayName="Registro" ref="A8:E40" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
+  <autoFilter ref="A8:E40" xr:uid="{F7E690B7-EC62-4BC2-A27A-E592475A3F24}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
@@ -1774,21 +1774,44 @@
         </is>
       </c>
     </row>
+    <row r="40" spans="1:5" ht="25.5" x14ac:dyDescent="0.35">
+      <c r="A40" s="11">
+        <v>46311</v>
+      </c>
+      <c r="B40" s="10" t="inlineStr">
+        <is>
+          <t>Pulizia della documentazione</t>
+        </is>
+      </c>
+      <c r="C40" s="12">
+        <v>0.5</v>
+      </c>
+      <c r="D40" s="9" t="inlineStr">
+        <is>
+          <t>Tolto il documento sulla verifica dei requisiti non funzionali, sostituito dall'elenco dei compiti, e ogni riferimento a MapTiler: la mappa usa solo Google Maps.</t>
+        </is>
+      </c>
+      <c r="E40" s="9" t="inlineStr">
+        <is>
+          <t>docs/fase-3-architettura-user-flow.md</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A7:E7"/>
   </mergeCells>
-  <conditionalFormatting sqref="C9:C39">
+  <conditionalFormatting sqref="C9:C40">
     <cfRule type="expression" dxfId="1" priority="1" stopIfTrue="1">
       <formula>($B9&lt;&gt;"")*($C9="")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Data non valida" error="Scrivi la data come gg/mm/aaaa, per esempio 14/10/2026." sqref="A9:A39" xr:uid="{D26B2BD8-0AFD-48FB-BBA1-B07F75408464}">
+    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Data non valida" error="Scrivi la data come gg/mm/aaaa, per esempio 14/10/2026." sqref="A9:A40" xr:uid="{D26B2BD8-0AFD-48FB-BBA1-B07F75408464}">
       <formula1>46023</formula1>
       <formula2>47483</formula2>
     </dataValidation>
-    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Ore non valide" error="Scrivi le ore come numero tra 0 e 24 (1,5 = un'ora e mezza)." promptTitle="Ore dedicate" prompt="Numero di ore, anche decimale: 1,5 = un'ora e mezza." sqref="C9:C39" xr:uid="{04EB0103-1D9C-4DFC-8906-92996DF6DE7A}">
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Ore non valide" error="Scrivi le ore come numero tra 0 e 24 (1,5 = un'ora e mezza)." promptTitle="Ore dedicate" prompt="Numero di ore, anche decimale: 1,5 = un'ora e mezza." sqref="C9:C40" xr:uid="{04EB0103-1D9C-4DFC-8906-92996DF6DE7A}">
       <formula1>0</formula1>
       <formula2>24</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
Aggiunge ai/test-0.1: prova di riconoscimento di due affreschi con DINOv2 small
Primo esperimento per lo scanner "Cosa sto guardando?" (RF-06), separato dal sito:
nessun file di versione-corrente è stato toccato.

- Script per calcolare l'impronta delle foto con DINOv2 small (Transformers.js), costruire
  l'indice, valutare con una prova onesta a blocchi e provare una foto nuova
- Report della prova su 72 foto di Casa Balduini e Palazzo Geremia: 72 su 72 giuste,
  62 su 62 con una sola foto di riferimento per luogo
- Le foto (con posizione GPS nell'EXIF), il modello e l'indice restano fuori da Git
- Voce nel libretto di Manuel

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/libretti/manuel-bulla.xlsx
+++ b/docs/libretti/manuel-bulla.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bulla\Documents\Ing-software-v1\docs\libretti\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB39AB5D-58FB-43A0-A16F-89E7ABB21BD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62583DCC-03D6-4C98-91A1-A5FB4026480C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{EB300ADB-58B5-479D-B51B-E912DFEACD78}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="117">
   <si>
     <t>Libretto delle attività</t>
   </si>
@@ -364,6 +364,36 @@
   </si>
   <si>
     <t>Nuovo controllo dopo le ultime modifiche (tedesco, satellite, galleria, sito online): 4 compiti chiusi, 3 nuovi, gli altri aggiornati; corretto il Riepilogo.</t>
+  </si>
+  <si>
+    <t>Riunione del team</t>
+  </si>
+  <si>
+    <t>Riunione con tutto il team per fare il punto sul progetto e decidere i prossimi compiti.</t>
+  </si>
+  <si>
+    <t>Mappa con Google Maps</t>
+  </si>
+  <si>
+    <t>Sfondo della mappa e vista satellitare con le tessere di Google Maps (Map Tiles API): chiave su Google Cloud limitata al dominio, ripiego su OpenStreetMap, informativa privacy e regole di sicurezza aggiornate.</t>
+  </si>
+  <si>
+    <t>versione-corrente/frontend/src/lib/sfondo.js</t>
+  </si>
+  <si>
+    <t>Pulizia della documentazione</t>
+  </si>
+  <si>
+    <t>Tolto il documento sulla verifica dei requisiti non funzionali, sostituito dall'elenco dei compiti, e ogni riferimento a MapTiler: la mappa usa solo Google Maps.</t>
+  </si>
+  <si>
+    <t>Test 0.1 del riconoscimento dei luoghi (DINOv2 small)</t>
+  </si>
+  <si>
+    <t>Scaricate le 72 foto di Marco da Drive e provato DINOv2 small a distinguere due affreschi: 72 su 72 giuste; provate anche due foto nuove.</t>
+  </si>
+  <si>
+    <t>ai/test-0.1/</t>
   </si>
 </sst>
 </file>
@@ -821,8 +851,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F7E690B7-EC62-4BC2-A27A-E592475A3F24}" name="Registro" displayName="Registro" ref="A8:E40" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
-  <autoFilter ref="A8:E40" xr:uid="{F7E690B7-EC62-4BC2-A27A-E592475A3F24}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F7E690B7-EC62-4BC2-A27A-E592475A3F24}" name="Registro" displayName="Registro" ref="A8:E41" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
+  <autoFilter ref="A8:E41" xr:uid="{F7E690B7-EC62-4BC2-A27A-E592475A3F24}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
@@ -1160,7 +1190,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.59765625" style="1" customWidth="1"/>
@@ -1197,7 +1227,7 @@
       </c>
       <c r="C5" s="7">
         <f>SUM(Registro[Ore])</f>
-        <v>43.5</v>
+        <v>51.5</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="13.15" x14ac:dyDescent="0.4">
@@ -1728,90 +1758,89 @@
         <v>80</v>
       </c>
     </row>
-    <row r="38" spans="1:5" ht="25.5" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:5" ht="13.15" x14ac:dyDescent="0.35">
       <c r="A38" s="11">
         <v>46311</v>
       </c>
-      <c r="B38" s="10" t="inlineStr">
-        <is>
-          <t>Riunione del team</t>
-        </is>
+      <c r="B38" s="10" t="s">
+        <v>107</v>
       </c>
       <c r="C38" s="12">
         <v>1</v>
       </c>
-      <c r="D38" s="9" t="inlineStr">
-        <is>
-          <t>Riunione con tutto il team per fare il punto sul progetto e decidere i prossimi compiti.</t>
-        </is>
-      </c>
-      <c r="E38" s="9" t="inlineStr">
-        <is>
-          <t>Riunione del team</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" spans="1:5" ht="25.5" x14ac:dyDescent="0.35">
+      <c r="D38" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="E38" s="9" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" ht="38.25" x14ac:dyDescent="0.35">
       <c r="A39" s="11">
         <v>46311</v>
       </c>
-      <c r="B39" s="10" t="inlineStr">
-        <is>
-          <t>Mappa con Google Maps</t>
-        </is>
+      <c r="B39" s="10" t="s">
+        <v>109</v>
       </c>
       <c r="C39" s="12">
         <v>3</v>
       </c>
-      <c r="D39" s="9" t="inlineStr">
-        <is>
-          <t>Sfondo della mappa e vista satellitare con le tessere di Google Maps (Map Tiles API): chiave su Google Cloud limitata al dominio, ripiego su OpenStreetMap, informativa privacy e regole di sicurezza aggiornate.</t>
-        </is>
-      </c>
-      <c r="E39" s="9" t="inlineStr">
-        <is>
-          <t>versione-corrente/frontend/src/lib/sfondo.js</t>
-        </is>
+      <c r="D39" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="E39" s="9" t="s">
+        <v>111</v>
       </c>
     </row>
     <row r="40" spans="1:5" ht="25.5" x14ac:dyDescent="0.35">
       <c r="A40" s="11">
         <v>46311</v>
       </c>
-      <c r="B40" s="10" t="inlineStr">
-        <is>
-          <t>Pulizia della documentazione</t>
-        </is>
+      <c r="B40" s="10" t="s">
+        <v>112</v>
       </c>
       <c r="C40" s="12">
         <v>0.5</v>
       </c>
-      <c r="D40" s="9" t="inlineStr">
-        <is>
-          <t>Tolto il documento sulla verifica dei requisiti non funzionali, sostituito dall'elenco dei compiti, e ogni riferimento a MapTiler: la mappa usa solo Google Maps.</t>
-        </is>
-      </c>
-      <c r="E40" s="9" t="inlineStr">
-        <is>
-          <t>docs/fase-3-architettura-user-flow.md</t>
-        </is>
+      <c r="D40" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="E40" s="9" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" ht="26.25" x14ac:dyDescent="0.35">
+      <c r="A41" s="11">
+        <v>46311</v>
+      </c>
+      <c r="B41" s="10" t="s">
+        <v>114</v>
+      </c>
+      <c r="C41" s="12">
+        <v>3.5</v>
+      </c>
+      <c r="D41" s="9" t="s">
+        <v>115</v>
+      </c>
+      <c r="E41" s="9" t="s">
+        <v>116</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A7:E7"/>
   </mergeCells>
-  <conditionalFormatting sqref="C9:C40">
+  <conditionalFormatting sqref="C9:C41">
     <cfRule type="expression" dxfId="1" priority="1" stopIfTrue="1">
       <formula>($B9&lt;&gt;"")*($C9="")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Data non valida" error="Scrivi la data come gg/mm/aaaa, per esempio 14/10/2026." sqref="A9:A40" xr:uid="{D26B2BD8-0AFD-48FB-BBA1-B07F75408464}">
+    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Data non valida" error="Scrivi la data come gg/mm/aaaa, per esempio 14/10/2026." sqref="A9:A41" xr:uid="{D26B2BD8-0AFD-48FB-BBA1-B07F75408464}">
       <formula1>46023</formula1>
       <formula2>47483</formula2>
     </dataValidation>
-    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Ore non valide" error="Scrivi le ore come numero tra 0 e 24 (1,5 = un'ora e mezza)." promptTitle="Ore dedicate" prompt="Numero di ore, anche decimale: 1,5 = un'ora e mezza." sqref="C9:C40" xr:uid="{04EB0103-1D9C-4DFC-8906-92996DF6DE7A}">
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Ore non valide" error="Scrivi le ore come numero tra 0 e 24 (1,5 = un'ora e mezza)." promptTitle="Ore dedicate" prompt="Numero di ore, anche decimale: 1,5 = un'ora e mezza." sqref="C9:C41" xr:uid="{04EB0103-1D9C-4DFC-8906-92996DF6DE7A}">
       <formula1>0</formula1>
       <formula2>24</formula2>
     </dataValidation>
@@ -1933,15 +1962,15 @@
       </c>
       <c r="C8" s="19">
         <f>COUNTIFS(Registro[Data],"&gt;="&amp;A8,Registro[Data],"&lt;="&amp;B8)</f>
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="D8" s="20">
         <f>SUMIFS(Registro[Ore],Registro[Data],"&gt;="&amp;A8,Registro[Data],"&lt;="&amp;B8)</f>
-        <v>17.5</v>
+        <v>25.5</v>
       </c>
       <c r="E8" s="20">
         <f>SUM(D$6:D8)</f>
-        <v>43.5</v>
+        <v>51.5</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
@@ -1963,7 +1992,7 @@
       </c>
       <c r="E9" s="23">
         <f>SUM(D$6:D9)</f>
-        <v>43.5</v>
+        <v>51.5</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
@@ -1985,7 +2014,7 @@
       </c>
       <c r="E10" s="20">
         <f>SUM(D$6:D10)</f>
-        <v>43.5</v>
+        <v>51.5</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.35">
@@ -2007,7 +2036,7 @@
       </c>
       <c r="E11" s="23">
         <f>SUM(D$6:D11)</f>
-        <v>43.5</v>
+        <v>51.5</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.35">
@@ -2029,7 +2058,7 @@
       </c>
       <c r="E12" s="20">
         <f>SUM(D$6:D12)</f>
-        <v>43.5</v>
+        <v>51.5</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
@@ -2051,7 +2080,7 @@
       </c>
       <c r="E13" s="23">
         <f>SUM(D$6:D13)</f>
-        <v>43.5</v>
+        <v>51.5</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
@@ -2073,7 +2102,7 @@
       </c>
       <c r="E14" s="20">
         <f>SUM(D$6:D14)</f>
-        <v>43.5</v>
+        <v>51.5</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.35">
@@ -2095,7 +2124,7 @@
       </c>
       <c r="E15" s="23">
         <f>SUM(D$6:D15)</f>
-        <v>43.5</v>
+        <v>51.5</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.35">
@@ -2117,7 +2146,7 @@
       </c>
       <c r="E16" s="20">
         <f>SUM(D$6:D16)</f>
-        <v>43.5</v>
+        <v>51.5</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.35">
@@ -2139,7 +2168,7 @@
       </c>
       <c r="E17" s="23">
         <f>SUM(D$6:D17)</f>
-        <v>43.5</v>
+        <v>51.5</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.35">
@@ -2161,7 +2190,7 @@
       </c>
       <c r="E18" s="20">
         <f>SUM(D$6:D18)</f>
-        <v>43.5</v>
+        <v>51.5</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.35">
@@ -2183,7 +2212,7 @@
       </c>
       <c r="E19" s="23">
         <f>SUM(D$6:D19)</f>
-        <v>43.5</v>
+        <v>51.5</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.35">
@@ -2205,7 +2234,7 @@
       </c>
       <c r="E20" s="20">
         <f>SUM(D$6:D20)</f>
-        <v>43.5</v>
+        <v>51.5</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.35">
@@ -2227,7 +2256,7 @@
       </c>
       <c r="E21" s="26">
         <f>SUM(D$6:D21)</f>
-        <v>43.5</v>
+        <v>51.5</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="13.15" x14ac:dyDescent="0.4">
@@ -2237,11 +2266,11 @@
       <c r="B22" s="28"/>
       <c r="C22" s="29">
         <f>SUM(C6:C21)</f>
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="D22" s="30">
         <f>SUM(D6:D21)</f>
-        <v>43.5</v>
+        <v>51.5</v>
       </c>
       <c r="E22" s="28"/>
     </row>
@@ -2253,7 +2282,7 @@
       <c r="C24" s="6"/>
       <c r="D24" s="15">
         <f>SUM(Registro[Ore])</f>
-        <v>43.5</v>
+        <v>51.5</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="13.15" x14ac:dyDescent="0.4">

</xml_diff>

<commit_message>
Aggiunge lo spot da 30 secondi del sito (bozza)
Spot animato di 30 secondi, 1280x720, con musica originale generata dal codice:
foto storica del Duomo, Palazzo Geremia, schermate del sito (mappa, schede,
itinerari, "Dov'era?") e schermata finale. Registrato con Chrome, senza programmi
esterni: ad.html contiene animazione e colonna sonora, registra.mjs produce il WebM
e la musica a parte, cattura.mjs prende le schermate dal sito online.

Voce nel libretto di Manuel.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/libretti/manuel-bulla.xlsx
+++ b/docs/libretti/manuel-bulla.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bulla\Documents\Ing-software-v1\docs\libretti\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62583DCC-03D6-4C98-91A1-A5FB4026480C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3CC7581-C183-4E7F-9F95-70A02EB201EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{EB300ADB-58B5-479D-B51B-E912DFEACD78}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="120">
   <si>
     <t>Libretto delle attività</t>
   </si>
@@ -394,6 +394,15 @@
   </si>
   <si>
     <t>ai/test-0.1/</t>
+  </si>
+  <si>
+    <t>Spot da 30 secondi del sito</t>
+  </si>
+  <si>
+    <t>Spot animato di 30 secondi con schermate del sito, foto d'epoca e musica originale, registrato in WebM con uno script.</t>
+  </si>
+  <si>
+    <t>presentazioni/ad-30s/</t>
   </si>
 </sst>
 </file>
@@ -851,8 +860,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F7E690B7-EC62-4BC2-A27A-E592475A3F24}" name="Registro" displayName="Registro" ref="A8:E41" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
-  <autoFilter ref="A8:E41" xr:uid="{F7E690B7-EC62-4BC2-A27A-E592475A3F24}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F7E690B7-EC62-4BC2-A27A-E592475A3F24}" name="Registro" displayName="Registro" ref="A8:E42" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
+  <autoFilter ref="A8:E42" xr:uid="{F7E690B7-EC62-4BC2-A27A-E592475A3F24}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
@@ -1190,7 +1199,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.59765625" style="1" customWidth="1"/>
@@ -1227,7 +1236,7 @@
       </c>
       <c r="C5" s="7">
         <f>SUM(Registro[Ore])</f>
-        <v>51.5</v>
+        <v>54.5</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="13.15" x14ac:dyDescent="0.4">
@@ -1826,21 +1835,38 @@
         <v>116</v>
       </c>
     </row>
+    <row r="42" spans="1:5" ht="25.5" x14ac:dyDescent="0.35">
+      <c r="A42" s="11">
+        <v>46311</v>
+      </c>
+      <c r="B42" s="10" t="s">
+        <v>117</v>
+      </c>
+      <c r="C42" s="12">
+        <v>3</v>
+      </c>
+      <c r="D42" s="9" t="s">
+        <v>118</v>
+      </c>
+      <c r="E42" s="9" t="s">
+        <v>119</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A7:E7"/>
   </mergeCells>
-  <conditionalFormatting sqref="C9:C41">
+  <conditionalFormatting sqref="C9:C42">
     <cfRule type="expression" dxfId="1" priority="1" stopIfTrue="1">
       <formula>($B9&lt;&gt;"")*($C9="")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Data non valida" error="Scrivi la data come gg/mm/aaaa, per esempio 14/10/2026." sqref="A9:A41" xr:uid="{D26B2BD8-0AFD-48FB-BBA1-B07F75408464}">
+    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Data non valida" error="Scrivi la data come gg/mm/aaaa, per esempio 14/10/2026." sqref="A9:A42" xr:uid="{D26B2BD8-0AFD-48FB-BBA1-B07F75408464}">
       <formula1>46023</formula1>
       <formula2>47483</formula2>
     </dataValidation>
-    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Ore non valide" error="Scrivi le ore come numero tra 0 e 24 (1,5 = un'ora e mezza)." promptTitle="Ore dedicate" prompt="Numero di ore, anche decimale: 1,5 = un'ora e mezza." sqref="C9:C41" xr:uid="{04EB0103-1D9C-4DFC-8906-92996DF6DE7A}">
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Ore non valide" error="Scrivi le ore come numero tra 0 e 24 (1,5 = un'ora e mezza)." promptTitle="Ore dedicate" prompt="Numero di ore, anche decimale: 1,5 = un'ora e mezza." sqref="C9:C42" xr:uid="{04EB0103-1D9C-4DFC-8906-92996DF6DE7A}">
       <formula1>0</formula1>
       <formula2>24</formula2>
     </dataValidation>
@@ -1962,15 +1988,15 @@
       </c>
       <c r="C8" s="19">
         <f>COUNTIFS(Registro[Data],"&gt;="&amp;A8,Registro[Data],"&lt;="&amp;B8)</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D8" s="20">
         <f>SUMIFS(Registro[Ore],Registro[Data],"&gt;="&amp;A8,Registro[Data],"&lt;="&amp;B8)</f>
-        <v>25.5</v>
+        <v>28.5</v>
       </c>
       <c r="E8" s="20">
         <f>SUM(D$6:D8)</f>
-        <v>51.5</v>
+        <v>54.5</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
@@ -1992,7 +2018,7 @@
       </c>
       <c r="E9" s="23">
         <f>SUM(D$6:D9)</f>
-        <v>51.5</v>
+        <v>54.5</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
@@ -2014,7 +2040,7 @@
       </c>
       <c r="E10" s="20">
         <f>SUM(D$6:D10)</f>
-        <v>51.5</v>
+        <v>54.5</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.35">
@@ -2036,7 +2062,7 @@
       </c>
       <c r="E11" s="23">
         <f>SUM(D$6:D11)</f>
-        <v>51.5</v>
+        <v>54.5</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.35">
@@ -2058,7 +2084,7 @@
       </c>
       <c r="E12" s="20">
         <f>SUM(D$6:D12)</f>
-        <v>51.5</v>
+        <v>54.5</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
@@ -2080,7 +2106,7 @@
       </c>
       <c r="E13" s="23">
         <f>SUM(D$6:D13)</f>
-        <v>51.5</v>
+        <v>54.5</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
@@ -2102,7 +2128,7 @@
       </c>
       <c r="E14" s="20">
         <f>SUM(D$6:D14)</f>
-        <v>51.5</v>
+        <v>54.5</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.35">
@@ -2124,7 +2150,7 @@
       </c>
       <c r="E15" s="23">
         <f>SUM(D$6:D15)</f>
-        <v>51.5</v>
+        <v>54.5</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.35">
@@ -2146,7 +2172,7 @@
       </c>
       <c r="E16" s="20">
         <f>SUM(D$6:D16)</f>
-        <v>51.5</v>
+        <v>54.5</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.35">
@@ -2168,7 +2194,7 @@
       </c>
       <c r="E17" s="23">
         <f>SUM(D$6:D17)</f>
-        <v>51.5</v>
+        <v>54.5</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.35">
@@ -2190,7 +2216,7 @@
       </c>
       <c r="E18" s="20">
         <f>SUM(D$6:D18)</f>
-        <v>51.5</v>
+        <v>54.5</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.35">
@@ -2212,7 +2238,7 @@
       </c>
       <c r="E19" s="23">
         <f>SUM(D$6:D19)</f>
-        <v>51.5</v>
+        <v>54.5</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.35">
@@ -2234,7 +2260,7 @@
       </c>
       <c r="E20" s="20">
         <f>SUM(D$6:D20)</f>
-        <v>51.5</v>
+        <v>54.5</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.35">
@@ -2256,7 +2282,7 @@
       </c>
       <c r="E21" s="26">
         <f>SUM(D$6:D21)</f>
-        <v>51.5</v>
+        <v>54.5</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="13.15" x14ac:dyDescent="0.4">
@@ -2266,11 +2292,11 @@
       <c r="B22" s="28"/>
       <c r="C22" s="29">
         <f>SUM(C6:C21)</f>
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D22" s="30">
         <f>SUM(D6:D21)</f>
-        <v>51.5</v>
+        <v>54.5</v>
       </c>
       <c r="E22" s="28"/>
     </row>
@@ -2282,7 +2308,7 @@
       <c r="C24" s="6"/>
       <c r="D24" s="15">
         <f>SUM(Registro[Ore])</f>
-        <v>51.5</v>
+        <v>54.5</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="13.15" x14ac:dyDescent="0.4">

</xml_diff>